<commit_message>
Remove explanatory notes from phase 1 materials
</commit_message>
<xml_diff>
--- a/Фаза 1 - Выбор концепции проекта/Фаза 1 Экспертные оценки.xlsx
+++ b/Фаза 1 - Выбор концепции проекта/Фаза 1 Экспертные оценки.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оценки" sheetId="1" r:id="Rdd7264972e244419"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOPSIS" sheetId="2" r:id="Rcf8ca93ff0ac4c1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="МАИ" sheetId="3" r:id="R86d215b3ab4e45f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итог" sheetId="4" r:id="R0550dfdf207f4035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оценки" sheetId="1" r:id="R96de4e6415fb4424"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOPSIS" sheetId="2" r:id="R2963168b361a4710"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="МАИ" sheetId="3" r:id="R6daa5d2c41904afc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итог" sheetId="4" r:id="Rf2f0280f27054ee1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -354,7 +354,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Имена экспертов указаны по составу команды; приведённые численные оценки сценарные, индивидуальный опрос не проводился.</x:v>
+        <x:v>Критерии, альтернативы и исходные оценки для сравнения концепций.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -5352,7 +5352,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>Оценки сценарные: индивидуальный опрос команды не проводился.</x:v>
+        <x:v>Промежуточные вычисления приведены на листах «TOPSIS» и «МАИ».</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add individual AHP consistency checks
</commit_message>
<xml_diff>
--- a/Фаза 1 - Выбор концепции проекта/Фаза 1 Экспертные оценки.xlsx
+++ b/Фаза 1 - Выбор концепции проекта/Фаза 1 Экспертные оценки.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оценки" sheetId="1" r:id="R96de4e6415fb4424"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOPSIS" sheetId="2" r:id="R2963168b361a4710"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="МАИ" sheetId="3" r:id="R6daa5d2c41904afc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итог" sheetId="4" r:id="Rf2f0280f27054ee1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Оценки" sheetId="1" r:id="R4471d1d5c89144d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOPSIS" sheetId="2" r:id="Rdc365f761d0f4a2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="МАИ" sheetId="3" r:id="Rb51ada5bd8ec446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итог" sheetId="4" r:id="R919fc2188ab6412d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3782,16 +3782,16 @@
         <x:v>Элемент</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
-        <x:v>C1 Полезность</x:v>
+        <x:v>C1</x:v>
       </x:c>
       <x:c r="C4" s="16" t="str">
-        <x:v>C2 Реализуемость</x:v>
+        <x:v>C2</x:v>
       </x:c>
       <x:c r="D4" s="16" t="str">
-        <x:v>C3 Ясность сценариев</x:v>
+        <x:v>C3</x:v>
       </x:c>
       <x:c r="E4" s="16" t="str">
-        <x:v>C4 Пригодность для планирования</x:v>
+        <x:v>C4</x:v>
       </x:c>
       <x:c r="F4" s="16" t="str">
         <x:v>Геом. ср.</x:v>
@@ -4027,16 +4027,16 @@
         <x:v>Элемент</x:v>
       </x:c>
       <x:c r="B14" s="17" t="str">
-        <x:v>A1 Бронирование помещений</x:v>
+        <x:v>A1</x:v>
       </x:c>
       <x:c r="C14" s="17" t="str">
-        <x:v>A2 Учебные группы</x:v>
+        <x:v>A2</x:v>
       </x:c>
       <x:c r="D14" s="17" t="str">
-        <x:v>A3 Студенческие события</x:v>
+        <x:v>A3</x:v>
       </x:c>
       <x:c r="E14" s="17" t="str">
-        <x:v>A4 Волонтёрские смены</x:v>
+        <x:v>A4</x:v>
       </x:c>
       <x:c r="F14" s="17" t="str">
         <x:v>Геом. ср.</x:v>
@@ -4272,16 +4272,16 @@
         <x:v>Элемент</x:v>
       </x:c>
       <x:c r="B24" s="17" t="str">
-        <x:v>A1 Бронирование помещений</x:v>
+        <x:v>A1</x:v>
       </x:c>
       <x:c r="C24" s="17" t="str">
-        <x:v>A2 Учебные группы</x:v>
+        <x:v>A2</x:v>
       </x:c>
       <x:c r="D24" s="17" t="str">
-        <x:v>A3 Студенческие события</x:v>
+        <x:v>A3</x:v>
       </x:c>
       <x:c r="E24" s="17" t="str">
-        <x:v>A4 Волонтёрские смены</x:v>
+        <x:v>A4</x:v>
       </x:c>
       <x:c r="F24" s="17" t="str">
         <x:v>Геом. ср.</x:v>
@@ -4517,16 +4517,16 @@
         <x:v>Элемент</x:v>
       </x:c>
       <x:c r="B34" s="17" t="str">
-        <x:v>A1 Бронирование помещений</x:v>
+        <x:v>A1</x:v>
       </x:c>
       <x:c r="C34" s="17" t="str">
-        <x:v>A2 Учебные группы</x:v>
+        <x:v>A2</x:v>
       </x:c>
       <x:c r="D34" s="17" t="str">
-        <x:v>A3 Студенческие события</x:v>
+        <x:v>A3</x:v>
       </x:c>
       <x:c r="E34" s="17" t="str">
-        <x:v>A4 Волонтёрские смены</x:v>
+        <x:v>A4</x:v>
       </x:c>
       <x:c r="F34" s="17" t="str">
         <x:v>Геом. ср.</x:v>
@@ -4762,16 +4762,16 @@
         <x:v>Элемент</x:v>
       </x:c>
       <x:c r="B44" s="17" t="str">
-        <x:v>A1 Бронирование помещений</x:v>
+        <x:v>A1</x:v>
       </x:c>
       <x:c r="C44" s="17" t="str">
-        <x:v>A2 Учебные группы</x:v>
+        <x:v>A2</x:v>
       </x:c>
       <x:c r="D44" s="17" t="str">
-        <x:v>A3 Студенческие события</x:v>
+        <x:v>A3</x:v>
       </x:c>
       <x:c r="E44" s="17" t="str">
-        <x:v>A4 Волонтёрские смены</x:v>
+        <x:v>A4</x:v>
       </x:c>
       <x:c r="F44" s="17" t="str">
         <x:v>Геом. ср.</x:v>
@@ -5160,6 +5160,4805 @@
       <x:c r="H59" s="13"/>
       <x:c r="I59" s="13"/>
     </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="4" t="str">
+        <x:v>Согласованность парных сравнений (CR &lt; 0,10)</x:v>
+      </x:c>
+      <x:c r="B62" s="4"/>
+      <x:c r="C62" s="4"/>
+      <x:c r="D62" s="4"/>
+      <x:c r="E62" s="4"/>
+      <x:c r="F62" s="4"/>
+      <x:c r="G62" s="4"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="8" t="str">
+        <x:v>Матрица</x:v>
+      </x:c>
+      <x:c r="B63" s="8" t="str">
+        <x:v>Роман Иванин</x:v>
+      </x:c>
+      <x:c r="C63" s="8" t="str">
+        <x:v>Баулин Евгений</x:v>
+      </x:c>
+      <x:c r="D63" s="8" t="str">
+        <x:v>Миленин Никита</x:v>
+      </x:c>
+      <x:c r="E63" s="8" t="str">
+        <x:v>Соу Мамаду</x:v>
+      </x:c>
+      <x:c r="F63" s="8" t="str">
+        <x:v>Группа</x:v>
+      </x:c>
+      <x:c r="G63" s="8" t="str">
+        <x:v>Макс. CR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>Критерии</x:v>
+      </x:c>
+      <x:c r="B64" s="5" t="n">
+        <x:f>I80</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C64" s="5" t="n">
+        <x:f>I90</x:f>
+        <x:v>0.003835657950578974</x:v>
+      </x:c>
+      <x:c r="D64" s="5" t="n">
+        <x:f>I100</x:f>
+        <x:v>0.003835657950578974</x:v>
+      </x:c>
+      <x:c r="E64" s="5" t="n">
+        <x:f>I110</x:f>
+        <x:v>0.007627513477776028</x:v>
+      </x:c>
+      <x:c r="F64" s="5" t="n">
+        <x:f>I11</x:f>
+        <x:v>0.0013907433679517646</x:v>
+      </x:c>
+      <x:c r="G64" s="5" t="n">
+        <x:f>MAX(B64:F64)</x:f>
+        <x:v>0.007627513477776028</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>C1 Полезность</x:v>
+      </x:c>
+      <x:c r="B65" s="5" t="n">
+        <x:f>I120</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+      <x:c r="C65" s="5" t="n">
+        <x:f>I130</x:f>
+        <x:v>0.01692292194386302</x:v>
+      </x:c>
+      <x:c r="D65" s="5" t="n">
+        <x:f>I140</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E65" s="5" t="n">
+        <x:f>I150</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+      <x:c r="F65" s="5" t="n">
+        <x:f>I21</x:f>
+        <x:v>0.01105452596306846</x:v>
+      </x:c>
+      <x:c r="G65" s="5" t="n">
+        <x:f>MAX(B65:F65)</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
+        <x:v>C2 Реализуемость</x:v>
+      </x:c>
+      <x:c r="B66" s="5" t="n">
+        <x:f>I160</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+      <x:c r="C66" s="5" t="n">
+        <x:f>I170</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+      <x:c r="D66" s="5" t="n">
+        <x:f>I180</x:f>
+        <x:v>0.003835657950579303</x:v>
+      </x:c>
+      <x:c r="E66" s="5" t="n">
+        <x:f>I190</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+      <x:c r="F66" s="5" t="n">
+        <x:f>I31</x:f>
+        <x:v>0.011535341011092909</x:v>
+      </x:c>
+      <x:c r="G66" s="5" t="n">
+        <x:f>MAX(B66:F66)</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
+        <x:v>C3 Ясность сценариев</x:v>
+      </x:c>
+      <x:c r="B67" s="5" t="n">
+        <x:f>I200</x:f>
+        <x:v>0.003835657950579303</x:v>
+      </x:c>
+      <x:c r="C67" s="5" t="n">
+        <x:f>I210</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+      <x:c r="D67" s="5" t="n">
+        <x:f>I220</x:f>
+        <x:v>0.007627513477775699</x:v>
+      </x:c>
+      <x:c r="E67" s="5" t="n">
+        <x:f>I230</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+      <x:c r="F67" s="5" t="n">
+        <x:f>I41</x:f>
+        <x:v>0.003979078518439039</x:v>
+      </x:c>
+      <x:c r="G67" s="5" t="n">
+        <x:f>MAX(B67:F67)</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>C4 Пригодность для планирования</x:v>
+      </x:c>
+      <x:c r="B68" s="5" t="n">
+        <x:f>I240</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+      <x:c r="C68" s="5" t="n">
+        <x:f>I250</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D68" s="5" t="n">
+        <x:f>I260</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+      <x:c r="E68" s="5" t="n">
+        <x:f>I270</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+      <x:c r="F68" s="5" t="n">
+        <x:f>I51</x:f>
+        <x:v>0.009499441785440878</x:v>
+      </x:c>
+      <x:c r="G68" s="5" t="n">
+        <x:f>MAX(B68:F68)</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="4" t="str">
+        <x:v>Критерии — Роман Иванин</x:v>
+      </x:c>
+      <x:c r="B72" s="4"/>
+      <x:c r="C72" s="4"/>
+      <x:c r="D72" s="4"/>
+      <x:c r="E72" s="4"/>
+      <x:c r="F72" s="4"/>
+      <x:c r="G72" s="4"/>
+      <x:c r="H72" s="4"/>
+      <x:c r="I72" s="4"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B73" s="8" t="str">
+        <x:v>C1</x:v>
+      </x:c>
+      <x:c r="C73" s="8" t="str">
+        <x:v>C2</x:v>
+      </x:c>
+      <x:c r="D73" s="8" t="str">
+        <x:v>C3</x:v>
+      </x:c>
+      <x:c r="E73" s="8" t="str">
+        <x:v>C4</x:v>
+      </x:c>
+      <x:c r="F73" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G73" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H73" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I73" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>C1 Полезность</x:v>
+      </x:c>
+      <x:c r="B74" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C74" s="5" t="n">
+        <x:f>'Оценки'!D41</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D74" s="5" t="n">
+        <x:f>'Оценки'!D42</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E74" s="5" t="n">
+        <x:f>'Оценки'!D43</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F74" s="5" t="n">
+        <x:f>PRODUCT(B74:E74)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G74" s="5" t="n">
+        <x:f>F74/SUM($F$74:$F$77)</x:f>
+        <x:v>0.28571428571428575</x:v>
+      </x:c>
+      <x:c r="H74" s="5" t="n">
+        <x:f>B74*$G$74+C74*$G$75+D74*$G$76+E74*$G$77</x:f>
+        <x:v>1.142857142857143</x:v>
+      </x:c>
+      <x:c r="I74" s="5" t="n">
+        <x:f>H74/G74</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>C2 Реализуемость</x:v>
+      </x:c>
+      <x:c r="B75" s="5" t="n">
+        <x:f>1/C74</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C75" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D75" s="5" t="n">
+        <x:f>'Оценки'!D44</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E75" s="5" t="n">
+        <x:f>'Оценки'!D45</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F75" s="5" t="n">
+        <x:f>PRODUCT(B75:E75)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G75" s="5" t="n">
+        <x:f>F75/SUM($F$74:$F$77)</x:f>
+        <x:v>0.28571428571428575</x:v>
+      </x:c>
+      <x:c r="H75" s="5" t="n">
+        <x:f>B75*$G$74+C75*$G$75+D75*$G$76+E75*$G$77</x:f>
+        <x:v>1.142857142857143</x:v>
+      </x:c>
+      <x:c r="I75" s="5" t="n">
+        <x:f>H75/G75</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>C3 Ясность сценариев</x:v>
+      </x:c>
+      <x:c r="B76" s="5" t="n">
+        <x:f>1/D74</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C76" s="5" t="n">
+        <x:f>1/D75</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D76" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E76" s="5" t="n">
+        <x:f>'Оценки'!D46</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F76" s="5" t="n">
+        <x:f>PRODUCT(B76:E76)^(1/4)</x:f>
+        <x:v>0.5946035575013605</x:v>
+      </x:c>
+      <x:c r="G76" s="5" t="n">
+        <x:f>F76/SUM($F$74:$F$77)</x:f>
+        <x:v>0.14285714285714288</x:v>
+      </x:c>
+      <x:c r="H76" s="5" t="n">
+        <x:f>B76*$G$74+C76*$G$75+D76*$G$76+E76*$G$77</x:f>
+        <x:v>0.5714285714285715</x:v>
+      </x:c>
+      <x:c r="I76" s="5" t="n">
+        <x:f>H76/G76</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>C4 Пригодность для планирования</x:v>
+      </x:c>
+      <x:c r="B77" s="5" t="n">
+        <x:f>1/E74</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C77" s="5" t="n">
+        <x:f>1/E75</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D77" s="5" t="n">
+        <x:f>1/E76</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E77" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F77" s="5" t="n">
+        <x:f>PRODUCT(B77:E77)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G77" s="5" t="n">
+        <x:f>F77/SUM($F$74:$F$77)</x:f>
+        <x:v>0.28571428571428575</x:v>
+      </x:c>
+      <x:c r="H77" s="5" t="n">
+        <x:f>B77*$G$74+C77*$G$75+D77*$G$76+E77*$G$77</x:f>
+        <x:v>1.142857142857143</x:v>
+      </x:c>
+      <x:c r="I77" s="5" t="n">
+        <x:f>H77/G77</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="B78" s="5"/>
+      <x:c r="C78" s="5"/>
+      <x:c r="D78" s="5"/>
+      <x:c r="E78" s="5"/>
+      <x:c r="F78" s="5"/>
+      <x:c r="G78" s="5"/>
+      <x:c r="H78" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I78" s="5" t="n">
+        <x:f>AVERAGE(I74:I77)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="B79" s="5"/>
+      <x:c r="C79" s="5"/>
+      <x:c r="D79" s="5"/>
+      <x:c r="E79" s="5"/>
+      <x:c r="F79" s="5"/>
+      <x:c r="G79" s="5"/>
+      <x:c r="H79" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I79" s="5" t="n">
+        <x:f>(I78-4)/3</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="B80" s="5"/>
+      <x:c r="C80" s="5"/>
+      <x:c r="D80" s="5"/>
+      <x:c r="E80" s="5"/>
+      <x:c r="F80" s="5"/>
+      <x:c r="G80" s="5"/>
+      <x:c r="H80" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I80" s="5" t="n">
+        <x:f>I79/0.9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="4" t="str">
+        <x:v>Критерии — Баулин Евгений</x:v>
+      </x:c>
+      <x:c r="B82" s="4"/>
+      <x:c r="C82" s="4"/>
+      <x:c r="D82" s="4"/>
+      <x:c r="E82" s="4"/>
+      <x:c r="F82" s="4"/>
+      <x:c r="G82" s="4"/>
+      <x:c r="H82" s="4"/>
+      <x:c r="I82" s="4"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B83" s="8" t="str">
+        <x:v>C1</x:v>
+      </x:c>
+      <x:c r="C83" s="8" t="str">
+        <x:v>C2</x:v>
+      </x:c>
+      <x:c r="D83" s="8" t="str">
+        <x:v>C3</x:v>
+      </x:c>
+      <x:c r="E83" s="8" t="str">
+        <x:v>C4</x:v>
+      </x:c>
+      <x:c r="F83" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G83" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H83" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I83" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>C1 Полезность</x:v>
+      </x:c>
+      <x:c r="B84" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C84" s="5" t="n">
+        <x:f>'Оценки'!E41</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D84" s="5" t="n">
+        <x:f>'Оценки'!E42</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E84" s="5" t="n">
+        <x:f>'Оценки'!E43</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F84" s="5" t="n">
+        <x:f>PRODUCT(B84:E84)^(1/4)</x:f>
+        <x:v>1.8612097182041991</x:v>
+      </x:c>
+      <x:c r="G84" s="5" t="n">
+        <x:f>F84/SUM($F$84:$F$87)</x:f>
+        <x:v>0.42314697456051914</x:v>
+      </x:c>
+      <x:c r="H84" s="5" t="n">
+        <x:f>B84*$G$84+C84*$G$85+D84*$G$86+E84*$G$87</x:f>
+        <x:v>1.6990050352741264</x:v>
+      </x:c>
+      <x:c r="I84" s="5" t="n">
+        <x:f>H84/G84</x:f>
+        <x:v>4.015165267431522</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>C2 Реализуемость</x:v>
+      </x:c>
+      <x:c r="B85" s="5" t="n">
+        <x:f>1/C84</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C85" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D85" s="5" t="n">
+        <x:f>'Оценки'!E44</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E85" s="5" t="n">
+        <x:f>'Оценки'!E45</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F85" s="5" t="n">
+        <x:f>PRODUCT(B85:E85)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G85" s="5" t="n">
+        <x:f>F85/SUM($F$84:$F$87)</x:f>
+        <x:v>0.22735050780241753</x:v>
+      </x:c>
+      <x:c r="H85" s="5" t="n">
+        <x:f>B85*$G$84+C85*$G$85+D85*$G$86+E85*$G$87</x:f>
+        <x:v>0.9105785225543861</x:v>
+      </x:c>
+      <x:c r="I85" s="5" t="n">
+        <x:f>H85/G85</x:f>
+        <x:v>4.005174790925642</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>C3 Ясность сценариев</x:v>
+      </x:c>
+      <x:c r="B86" s="5" t="n">
+        <x:f>1/D84</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="C86" s="5" t="n">
+        <x:f>1/D85</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D86" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E86" s="5" t="n">
+        <x:f>'Оценки'!E46</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F86" s="5" t="n">
+        <x:f>PRODUCT(B86:E86)^(1/4)</x:f>
+        <x:v>0.537284965911771</x:v>
+      </x:c>
+      <x:c r="G86" s="5" t="n">
+        <x:f>F86/SUM($F$84:$F$87)</x:f>
+        <x:v>0.12215200983464573</x:v>
+      </x:c>
+      <x:c r="H86" s="5" t="n">
+        <x:f>B86*$G$84+C86*$G$85+D86*$G$86+E86*$G$87</x:f>
+        <x:v>0.4905515091572363</x:v>
+      </x:c>
+      <x:c r="I86" s="5" t="n">
+        <x:f>H86/G86</x:f>
+        <x:v>4.01591025658345</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>C4 Пригодность для планирования</x:v>
+      </x:c>
+      <x:c r="B87" s="5" t="n">
+        <x:f>1/E84</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C87" s="5" t="n">
+        <x:f>1/E85</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D87" s="5" t="n">
+        <x:f>1/E86</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E87" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F87" s="5" t="n">
+        <x:f>PRODUCT(B87:E87)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G87" s="5" t="n">
+        <x:f>F87/SUM($F$84:$F$87)</x:f>
+        <x:v>0.22735050780241753</x:v>
+      </x:c>
+      <x:c r="H87" s="5" t="n">
+        <x:f>B87*$G$84+C87*$G$85+D87*$G$86+E87*$G$87</x:f>
+        <x:v>0.9105785225543861</x:v>
+      </x:c>
+      <x:c r="I87" s="5" t="n">
+        <x:f>H87/G87</x:f>
+        <x:v>4.005174790925642</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="B88" s="5"/>
+      <x:c r="C88" s="5"/>
+      <x:c r="D88" s="5"/>
+      <x:c r="E88" s="5"/>
+      <x:c r="F88" s="5"/>
+      <x:c r="G88" s="5"/>
+      <x:c r="H88" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I88" s="5" t="n">
+        <x:f>AVERAGE(I84:I87)</x:f>
+        <x:v>4.010356276466563</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="B89" s="5"/>
+      <x:c r="C89" s="5"/>
+      <x:c r="D89" s="5"/>
+      <x:c r="E89" s="5"/>
+      <x:c r="F89" s="5"/>
+      <x:c r="G89" s="5"/>
+      <x:c r="H89" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I89" s="5" t="n">
+        <x:f>(I88-4)/3</x:f>
+        <x:v>0.003452092155521077</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="B90" s="5"/>
+      <x:c r="C90" s="5"/>
+      <x:c r="D90" s="5"/>
+      <x:c r="E90" s="5"/>
+      <x:c r="F90" s="5"/>
+      <x:c r="G90" s="5"/>
+      <x:c r="H90" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I90" s="5" t="n">
+        <x:f>I89/0.9</x:f>
+        <x:v>0.003835657950578974</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="4" t="str">
+        <x:v>Критерии — Миленин Никита</x:v>
+      </x:c>
+      <x:c r="B92" s="4"/>
+      <x:c r="C92" s="4"/>
+      <x:c r="D92" s="4"/>
+      <x:c r="E92" s="4"/>
+      <x:c r="F92" s="4"/>
+      <x:c r="G92" s="4"/>
+      <x:c r="H92" s="4"/>
+      <x:c r="I92" s="4"/>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B93" s="8" t="str">
+        <x:v>C1</x:v>
+      </x:c>
+      <x:c r="C93" s="8" t="str">
+        <x:v>C2</x:v>
+      </x:c>
+      <x:c r="D93" s="8" t="str">
+        <x:v>C3</x:v>
+      </x:c>
+      <x:c r="E93" s="8" t="str">
+        <x:v>C4</x:v>
+      </x:c>
+      <x:c r="F93" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G93" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H93" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I93" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>C1 Полезность</x:v>
+      </x:c>
+      <x:c r="B94" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C94" s="5" t="n">
+        <x:f>'Оценки'!F41</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D94" s="5" t="n">
+        <x:f>'Оценки'!F42</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E94" s="5" t="n">
+        <x:f>'Оценки'!F43</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F94" s="5" t="n">
+        <x:f>PRODUCT(B94:E94)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G94" s="5" t="n">
+        <x:f>F94/SUM($F$94:$F$97)</x:f>
+        <x:v>0.22735050780241753</x:v>
+      </x:c>
+      <x:c r="H94" s="5" t="n">
+        <x:f>B94*$G$94+C94*$G$95+D94*$G$96+E94*$G$97</x:f>
+        <x:v>0.9105785225543861</x:v>
+      </x:c>
+      <x:c r="I94" s="5" t="n">
+        <x:f>H94/G94</x:f>
+        <x:v>4.005174790925642</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>C2 Реализуемость</x:v>
+      </x:c>
+      <x:c r="B95" s="5" t="n">
+        <x:f>1/C94</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C95" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D95" s="5" t="n">
+        <x:f>'Оценки'!F44</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E95" s="5" t="n">
+        <x:f>'Оценки'!F45</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F95" s="5" t="n">
+        <x:f>PRODUCT(B95:E95)^(1/4)</x:f>
+        <x:v>1.8612097182041991</x:v>
+      </x:c>
+      <x:c r="G95" s="5" t="n">
+        <x:f>F95/SUM($F$94:$F$97)</x:f>
+        <x:v>0.42314697456051914</x:v>
+      </x:c>
+      <x:c r="H95" s="5" t="n">
+        <x:f>B95*$G$94+C95*$G$95+D95*$G$96+E95*$G$97</x:f>
+        <x:v>1.6990050352741264</x:v>
+      </x:c>
+      <x:c r="I95" s="5" t="n">
+        <x:f>H95/G95</x:f>
+        <x:v>4.015165267431522</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>C3 Ясность сценариев</x:v>
+      </x:c>
+      <x:c r="B96" s="5" t="n">
+        <x:f>1/D94</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C96" s="5" t="n">
+        <x:f>1/D95</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="D96" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E96" s="5" t="n">
+        <x:f>'Оценки'!F46</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F96" s="5" t="n">
+        <x:f>PRODUCT(B96:E96)^(1/4)</x:f>
+        <x:v>0.537284965911771</x:v>
+      </x:c>
+      <x:c r="G96" s="5" t="n">
+        <x:f>F96/SUM($F$94:$F$97)</x:f>
+        <x:v>0.12215200983464573</x:v>
+      </x:c>
+      <x:c r="H96" s="5" t="n">
+        <x:f>B96*$G$94+C96*$G$95+D96*$G$96+E96*$G$97</x:f>
+        <x:v>0.4905515091572363</x:v>
+      </x:c>
+      <x:c r="I96" s="5" t="n">
+        <x:f>H96/G96</x:f>
+        <x:v>4.01591025658345</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>C4 Пригодность для планирования</x:v>
+      </x:c>
+      <x:c r="B97" s="5" t="n">
+        <x:f>1/E94</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C97" s="5" t="n">
+        <x:f>1/E95</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D97" s="5" t="n">
+        <x:f>1/E96</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E97" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F97" s="5" t="n">
+        <x:f>PRODUCT(B97:E97)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G97" s="5" t="n">
+        <x:f>F97/SUM($F$94:$F$97)</x:f>
+        <x:v>0.22735050780241753</x:v>
+      </x:c>
+      <x:c r="H97" s="5" t="n">
+        <x:f>B97*$G$94+C97*$G$95+D97*$G$96+E97*$G$97</x:f>
+        <x:v>0.9105785225543861</x:v>
+      </x:c>
+      <x:c r="I97" s="5" t="n">
+        <x:f>H97/G97</x:f>
+        <x:v>4.005174790925642</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="B98" s="5"/>
+      <x:c r="C98" s="5"/>
+      <x:c r="D98" s="5"/>
+      <x:c r="E98" s="5"/>
+      <x:c r="F98" s="5"/>
+      <x:c r="G98" s="5"/>
+      <x:c r="H98" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I98" s="5" t="n">
+        <x:f>AVERAGE(I94:I97)</x:f>
+        <x:v>4.010356276466563</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="B99" s="5"/>
+      <x:c r="C99" s="5"/>
+      <x:c r="D99" s="5"/>
+      <x:c r="E99" s="5"/>
+      <x:c r="F99" s="5"/>
+      <x:c r="G99" s="5"/>
+      <x:c r="H99" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I99" s="5" t="n">
+        <x:f>(I98-4)/3</x:f>
+        <x:v>0.003452092155521077</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="B100" s="5"/>
+      <x:c r="C100" s="5"/>
+      <x:c r="D100" s="5"/>
+      <x:c r="E100" s="5"/>
+      <x:c r="F100" s="5"/>
+      <x:c r="G100" s="5"/>
+      <x:c r="H100" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I100" s="5" t="n">
+        <x:f>I99/0.9</x:f>
+        <x:v>0.003835657950578974</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="4" t="str">
+        <x:v>Критерии — Соу Мамаду</x:v>
+      </x:c>
+      <x:c r="B102" s="4"/>
+      <x:c r="C102" s="4"/>
+      <x:c r="D102" s="4"/>
+      <x:c r="E102" s="4"/>
+      <x:c r="F102" s="4"/>
+      <x:c r="G102" s="4"/>
+      <x:c r="H102" s="4"/>
+      <x:c r="I102" s="4"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B103" s="8" t="str">
+        <x:v>C1</x:v>
+      </x:c>
+      <x:c r="C103" s="8" t="str">
+        <x:v>C2</x:v>
+      </x:c>
+      <x:c r="D103" s="8" t="str">
+        <x:v>C3</x:v>
+      </x:c>
+      <x:c r="E103" s="8" t="str">
+        <x:v>C4</x:v>
+      </x:c>
+      <x:c r="F103" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G103" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H103" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I103" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="str">
+        <x:v>C1 Полезность</x:v>
+      </x:c>
+      <x:c r="B104" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C104" s="5" t="n">
+        <x:f>'Оценки'!G41</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D104" s="5" t="n">
+        <x:f>'Оценки'!G42</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E104" s="5" t="n">
+        <x:f>'Оценки'!G43</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F104" s="5" t="n">
+        <x:f>PRODUCT(B104:E104)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G104" s="5" t="n">
+        <x:f>F104/SUM($F$104:$F$107)</x:f>
+        <x:v>0.28101863127026006</x:v>
+      </x:c>
+      <x:c r="H104" s="5" t="n">
+        <x:f>B104*$G$104+C104*$G$105+D104*$G$106+E104*$G$107</x:f>
+        <x:v>1.1269644991337515</x:v>
+      </x:c>
+      <x:c r="I104" s="5" t="n">
+        <x:f>H104/G104</x:f>
+        <x:v>4.010283923310166</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="str">
+        <x:v>C2 Реализуемость</x:v>
+      </x:c>
+      <x:c r="B105" s="5" t="n">
+        <x:f>1/C104</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C105" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D105" s="5" t="n">
+        <x:f>'Оценки'!G44</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E105" s="5" t="n">
+        <x:f>'Оценки'!G45</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F105" s="5" t="n">
+        <x:f>PRODUCT(B105:E105)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G105" s="5" t="n">
+        <x:f>F105/SUM($F$104:$F$107)</x:f>
+        <x:v>0.28101863127026006</x:v>
+      </x:c>
+      <x:c r="H105" s="5" t="n">
+        <x:f>B105*$G$104+C105*$G$105+D105*$G$106+E105*$G$107</x:f>
+        <x:v>1.1269644991337515</x:v>
+      </x:c>
+      <x:c r="I105" s="5" t="n">
+        <x:f>H105/G105</x:f>
+        <x:v>4.010283923310166</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="str">
+        <x:v>C3 Ясность сценариев</x:v>
+      </x:c>
+      <x:c r="B106" s="5" t="n">
+        <x:f>1/D104</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C106" s="5" t="n">
+        <x:f>1/D105</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D106" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E106" s="5" t="n">
+        <x:f>'Оценки'!G46</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="F106" s="5" t="n">
+        <x:f>PRODUCT(B106:E106)^(1/4)</x:f>
+        <x:v>0.537284965911771</x:v>
+      </x:c>
+      <x:c r="G106" s="5" t="n">
+        <x:f>F106/SUM($F$104:$F$107)</x:f>
+        <x:v>0.1269644991337516</x:v>
+      </x:c>
+      <x:c r="H106" s="5" t="n">
+        <x:f>B106*$G$104+C106*$G$105+D106*$G$106+E106*$G$107</x:f>
+        <x:v>0.5116492098459211</x:v>
+      </x:c>
+      <x:c r="I106" s="5" t="n">
+        <x:f>H106/G106</x:f>
+        <x:v>4.02986042032837</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="str">
+        <x:v>C4 Пригодность для планирования</x:v>
+      </x:c>
+      <x:c r="B107" s="5" t="n">
+        <x:f>1/E104</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C107" s="5" t="n">
+        <x:f>1/E105</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D107" s="5" t="n">
+        <x:f>1/E106</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E107" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F107" s="5" t="n">
+        <x:f>PRODUCT(B107:E107)^(1/4)</x:f>
+        <x:v>1.3160740129524924</x:v>
+      </x:c>
+      <x:c r="G107" s="5" t="n">
+        <x:f>F107/SUM($F$104:$F$107)</x:f>
+        <x:v>0.3109982383257282</x:v>
+      </x:c>
+      <x:c r="H107" s="5" t="n">
+        <x:f>B107*$G$104+C107*$G$105+D107*$G$106+E107*$G$107</x:f>
+        <x:v>1.253928998267503</x:v>
+      </x:c>
+      <x:c r="I107" s="5" t="n">
+        <x:f>H107/G107</x:f>
+        <x:v>4.031948878611279</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="B108" s="5"/>
+      <x:c r="C108" s="5"/>
+      <x:c r="D108" s="5"/>
+      <x:c r="E108" s="5"/>
+      <x:c r="F108" s="5"/>
+      <x:c r="G108" s="5"/>
+      <x:c r="H108" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I108" s="5" t="n">
+        <x:f>AVERAGE(I104:I107)</x:f>
+        <x:v>4.020594286389995</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="B109" s="5"/>
+      <x:c r="C109" s="5"/>
+      <x:c r="D109" s="5"/>
+      <x:c r="E109" s="5"/>
+      <x:c r="F109" s="5"/>
+      <x:c r="G109" s="5"/>
+      <x:c r="H109" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I109" s="5" t="n">
+        <x:f>(I108-4)/3</x:f>
+        <x:v>0.006864762129998425</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="B110" s="5"/>
+      <x:c r="C110" s="5"/>
+      <x:c r="D110" s="5"/>
+      <x:c r="E110" s="5"/>
+      <x:c r="F110" s="5"/>
+      <x:c r="G110" s="5"/>
+      <x:c r="H110" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I110" s="5" t="n">
+        <x:f>I109/0.9</x:f>
+        <x:v>0.007627513477776028</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="4" t="str">
+        <x:v>C1 Полезность — Роман Иванин</x:v>
+      </x:c>
+      <x:c r="B112" s="4"/>
+      <x:c r="C112" s="4"/>
+      <x:c r="D112" s="4"/>
+      <x:c r="E112" s="4"/>
+      <x:c r="F112" s="4"/>
+      <x:c r="G112" s="4"/>
+      <x:c r="H112" s="4"/>
+      <x:c r="I112" s="4"/>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B113" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C113" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D113" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E113" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F113" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G113" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H113" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I113" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B114" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C114" s="5" t="n">
+        <x:f>'Оценки'!D47</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D114" s="5" t="n">
+        <x:f>'Оценки'!D48</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E114" s="5" t="n">
+        <x:f>'Оценки'!D49</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F114" s="5" t="n">
+        <x:f>PRODUCT(B114:E114)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G114" s="5" t="n">
+        <x:f>F114/SUM($F$114:$F$117)</x:f>
+        <x:v>0.20529665596111354</x:v>
+      </x:c>
+      <x:c r="H114" s="5" t="n">
+        <x:f>B114*$G$114+C114*$G$115+D114*$G$116+E114*$G$117</x:f>
+        <x:v>0.8273667779387246</x:v>
+      </x:c>
+      <x:c r="I114" s="5" t="n">
+        <x:f>H114/G114</x:f>
+        <x:v>4.030103530256436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B115" s="5" t="n">
+        <x:f>1/C114</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C115" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D115" s="5" t="n">
+        <x:f>'Оценки'!D50</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E115" s="5" t="n">
+        <x:f>'Оценки'!D51</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F115" s="5" t="n">
+        <x:f>PRODUCT(B115:E115)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G115" s="5" t="n">
+        <x:f>F115/SUM($F$114:$F$117)</x:f>
+        <x:v>0.20529665596111354</x:v>
+      </x:c>
+      <x:c r="H115" s="5" t="n">
+        <x:f>B115*$G$114+C115*$G$115+D115*$G$116+E115*$G$117</x:f>
+        <x:v>0.8273667779387246</x:v>
+      </x:c>
+      <x:c r="I115" s="5" t="n">
+        <x:f>H115/G115</x:f>
+        <x:v>4.030103530256436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B116" s="5" t="n">
+        <x:f>1/D114</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C116" s="5" t="n">
+        <x:f>1/D115</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D116" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E116" s="5" t="n">
+        <x:f>'Оценки'!D52</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F116" s="5" t="n">
+        <x:f>PRODUCT(B116:E116)^(1/4)</x:f>
+        <x:v>1.4142135623730951</x:v>
+      </x:c>
+      <x:c r="G116" s="5" t="n">
+        <x:f>F116/SUM($F$114:$F$117)</x:f>
+        <x:v>0.34526644412255103</x:v>
+      </x:c>
+      <x:c r="H116" s="5" t="n">
+        <x:f>B116*$G$114+C116*$G$115+D116*$G$116+E116*$G$117</x:f>
+        <x:v>1.4105933119222271</x:v>
+      </x:c>
+      <x:c r="I116" s="5" t="n">
+        <x:f>H116/G116</x:f>
+        <x:v>4.0855210111919895</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B117" s="5" t="n">
+        <x:f>1/E114</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C117" s="5" t="n">
+        <x:f>1/E115</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D117" s="5" t="n">
+        <x:f>1/E116</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E117" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F117" s="5" t="n">
+        <x:f>PRODUCT(B117:E117)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G117" s="5" t="n">
+        <x:f>F117/SUM($F$114:$F$117)</x:f>
+        <x:v>0.24414024395522202</x:v>
+      </x:c>
+      <x:c r="H117" s="5" t="n">
+        <x:f>B117*$G$114+C117*$G$115+D117*$G$116+E117*$G$117</x:f>
+        <x:v>1.0000000000000002</x:v>
+      </x:c>
+      <x:c r="I117" s="5" t="n">
+        <x:f>H117/G117</x:f>
+        <x:v>4.096006392880525</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="B118" s="5"/>
+      <x:c r="C118" s="5"/>
+      <x:c r="D118" s="5"/>
+      <x:c r="E118" s="5"/>
+      <x:c r="F118" s="5"/>
+      <x:c r="G118" s="5"/>
+      <x:c r="H118" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I118" s="5" t="n">
+        <x:f>AVERAGE(I114:I117)</x:f>
+        <x:v>4.060433616146346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="B119" s="5"/>
+      <x:c r="C119" s="5"/>
+      <x:c r="D119" s="5"/>
+      <x:c r="E119" s="5"/>
+      <x:c r="F119" s="5"/>
+      <x:c r="G119" s="5"/>
+      <x:c r="H119" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I119" s="5" t="n">
+        <x:f>(I118-4)/3</x:f>
+        <x:v>0.020144538715448707</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="B120" s="5"/>
+      <x:c r="C120" s="5"/>
+      <x:c r="D120" s="5"/>
+      <x:c r="E120" s="5"/>
+      <x:c r="F120" s="5"/>
+      <x:c r="G120" s="5"/>
+      <x:c r="H120" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I120" s="5" t="n">
+        <x:f>I119/0.9</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="4" t="str">
+        <x:v>C1 Полезность — Баулин Евгений</x:v>
+      </x:c>
+      <x:c r="B122" s="4"/>
+      <x:c r="C122" s="4"/>
+      <x:c r="D122" s="4"/>
+      <x:c r="E122" s="4"/>
+      <x:c r="F122" s="4"/>
+      <x:c r="G122" s="4"/>
+      <x:c r="H122" s="4"/>
+      <x:c r="I122" s="4"/>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B123" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C123" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D123" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E123" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F123" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G123" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H123" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I123" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B124" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C124" s="5" t="n">
+        <x:f>'Оценки'!E47</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D124" s="5" t="n">
+        <x:f>'Оценки'!E48</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="E124" s="5" t="n">
+        <x:f>'Оценки'!E49</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F124" s="5" t="n">
+        <x:f>PRODUCT(B124:E124)^(1/4)</x:f>
+        <x:v>0.537284965911771</x:v>
+      </x:c>
+      <x:c r="G124" s="5" t="n">
+        <x:f>F124/SUM($F$124:$F$127)</x:f>
+        <x:v>0.1251952390355543</x:v>
+      </x:c>
+      <x:c r="H124" s="5" t="n">
+        <x:f>B124*$G$124+C124*$G$125+D124*$G$126+E124*$G$127</x:f>
+        <x:v>0.501816361109084</x:v>
+      </x:c>
+      <x:c r="I124" s="5" t="n">
+        <x:f>H124/G124</x:f>
+        <x:v>4.008270322217068</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B125" s="5" t="n">
+        <x:f>1/C124</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C125" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D125" s="5" t="n">
+        <x:f>'Оценки'!E50</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E125" s="5" t="n">
+        <x:f>'Оценки'!E51</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F125" s="5" t="n">
+        <x:f>PRODUCT(B125:E125)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G125" s="5" t="n">
+        <x:f>F125/SUM($F$124:$F$127)</x:f>
+        <x:v>0.23301459556587137</x:v>
+      </x:c>
+      <x:c r="H125" s="5" t="n">
+        <x:f>B125*$G$124+C125*$G$125+D125*$G$126+E125*$G$127</x:f>
+        <x:v>0.9428514638094749</x:v>
+      </x:c>
+      <x:c r="I125" s="5" t="n">
+        <x:f>H125/G125</x:f>
+        <x:v>4.046319336862906</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B126" s="5" t="n">
+        <x:f>1/D124</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C126" s="5" t="n">
+        <x:f>1/D125</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D126" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E126" s="5" t="n">
+        <x:f>'Оценки'!E52</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F126" s="5" t="n">
+        <x:f>PRODUCT(B126:E126)^(1/4)</x:f>
+        <x:v>1.5650845800732873</x:v>
+      </x:c>
+      <x:c r="G126" s="5" t="n">
+        <x:f>F126/SUM($F$124:$F$127)</x:f>
+        <x:v>0.36468755045215867</x:v>
+      </x:c>
+      <x:c r="H126" s="5" t="n">
+        <x:f>B126*$G$124+C126*$G$125+D126*$G$126+E126*$G$127</x:f>
+        <x:v>1.4834050736369802</x:v>
+      </x:c>
+      <x:c r="I126" s="5" t="n">
+        <x:f>H126/G126</x:f>
+        <x:v>4.067605466097697</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B127" s="5" t="n">
+        <x:f>1/E124</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C127" s="5" t="n">
+        <x:f>1/E125</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D127" s="5" t="n">
+        <x:f>1/E126</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E127" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F127" s="5" t="n">
+        <x:f>PRODUCT(B127:E127)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G127" s="5" t="n">
+        <x:f>F127/SUM($F$124:$F$127)</x:f>
+        <x:v>0.2771026149464157</x:v>
+      </x:c>
+      <x:c r="H127" s="5" t="n">
+        <x:f>B127*$G$124+C127*$G$125+D127*$G$126+E127*$G$127</x:f>
+        <x:v>1.1251952390355544</x:v>
+      </x:c>
+      <x:c r="I127" s="5" t="n">
+        <x:f>H127/G127</x:f>
+        <x:v>4.060572431816053</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="B128" s="5"/>
+      <x:c r="C128" s="5"/>
+      <x:c r="D128" s="5"/>
+      <x:c r="E128" s="5"/>
+      <x:c r="F128" s="5"/>
+      <x:c r="G128" s="5"/>
+      <x:c r="H128" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I128" s="5" t="n">
+        <x:f>AVERAGE(I124:I127)</x:f>
+        <x:v>4.04569188924843</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="B129" s="5"/>
+      <x:c r="C129" s="5"/>
+      <x:c r="D129" s="5"/>
+      <x:c r="E129" s="5"/>
+      <x:c r="F129" s="5"/>
+      <x:c r="G129" s="5"/>
+      <x:c r="H129" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I129" s="5" t="n">
+        <x:f>(I128-4)/3</x:f>
+        <x:v>0.015230629749476718</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="B130" s="5"/>
+      <x:c r="C130" s="5"/>
+      <x:c r="D130" s="5"/>
+      <x:c r="E130" s="5"/>
+      <x:c r="F130" s="5"/>
+      <x:c r="G130" s="5"/>
+      <x:c r="H130" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I130" s="5" t="n">
+        <x:f>I129/0.9</x:f>
+        <x:v>0.01692292194386302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="4" t="str">
+        <x:v>C1 Полезность — Миленин Никита</x:v>
+      </x:c>
+      <x:c r="B132" s="4"/>
+      <x:c r="C132" s="4"/>
+      <x:c r="D132" s="4"/>
+      <x:c r="E132" s="4"/>
+      <x:c r="F132" s="4"/>
+      <x:c r="G132" s="4"/>
+      <x:c r="H132" s="4"/>
+      <x:c r="I132" s="4"/>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B133" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C133" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D133" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E133" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F133" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G133" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H133" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I133" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B134" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C134" s="5" t="n">
+        <x:f>'Оценки'!F47</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D134" s="5" t="n">
+        <x:f>'Оценки'!F48</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E134" s="5" t="n">
+        <x:f>'Оценки'!F49</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F134" s="5" t="n">
+        <x:f>PRODUCT(B134:E134)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G134" s="5" t="n">
+        <x:f>F134/SUM($F$134:$F$137)</x:f>
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="H134" s="5" t="n">
+        <x:f>B134*$G$134+C134*$G$135+D134*$G$136+E134*$G$137</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I134" s="5" t="n">
+        <x:f>H134/G134</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B135" s="5" t="n">
+        <x:f>1/C134</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C135" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D135" s="5" t="n">
+        <x:f>'Оценки'!F50</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E135" s="5" t="n">
+        <x:f>'Оценки'!F51</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F135" s="5" t="n">
+        <x:f>PRODUCT(B135:E135)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G135" s="5" t="n">
+        <x:f>F135/SUM($F$134:$F$137)</x:f>
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="H135" s="5" t="n">
+        <x:f>B135*$G$134+C135*$G$135+D135*$G$136+E135*$G$137</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I135" s="5" t="n">
+        <x:f>H135/G135</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B136" s="5" t="n">
+        <x:f>1/D134</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C136" s="5" t="n">
+        <x:f>1/D135</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D136" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E136" s="5" t="n">
+        <x:f>'Оценки'!F52</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F136" s="5" t="n">
+        <x:f>PRODUCT(B136:E136)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G136" s="5" t="n">
+        <x:f>F136/SUM($F$134:$F$137)</x:f>
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="H136" s="5" t="n">
+        <x:f>B136*$G$134+C136*$G$135+D136*$G$136+E136*$G$137</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I136" s="5" t="n">
+        <x:f>H136/G136</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B137" s="5" t="n">
+        <x:f>1/E134</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C137" s="5" t="n">
+        <x:f>1/E135</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D137" s="5" t="n">
+        <x:f>1/E136</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E137" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F137" s="5" t="n">
+        <x:f>PRODUCT(B137:E137)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G137" s="5" t="n">
+        <x:f>F137/SUM($F$134:$F$137)</x:f>
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="H137" s="5" t="n">
+        <x:f>B137*$G$134+C137*$G$135+D137*$G$136+E137*$G$137</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I137" s="5" t="n">
+        <x:f>H137/G137</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="B138" s="5"/>
+      <x:c r="C138" s="5"/>
+      <x:c r="D138" s="5"/>
+      <x:c r="E138" s="5"/>
+      <x:c r="F138" s="5"/>
+      <x:c r="G138" s="5"/>
+      <x:c r="H138" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I138" s="5" t="n">
+        <x:f>AVERAGE(I134:I137)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="B139" s="5"/>
+      <x:c r="C139" s="5"/>
+      <x:c r="D139" s="5"/>
+      <x:c r="E139" s="5"/>
+      <x:c r="F139" s="5"/>
+      <x:c r="G139" s="5"/>
+      <x:c r="H139" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I139" s="5" t="n">
+        <x:f>(I138-4)/3</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="B140" s="5"/>
+      <x:c r="C140" s="5"/>
+      <x:c r="D140" s="5"/>
+      <x:c r="E140" s="5"/>
+      <x:c r="F140" s="5"/>
+      <x:c r="G140" s="5"/>
+      <x:c r="H140" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I140" s="5" t="n">
+        <x:f>I139/0.9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="4" t="str">
+        <x:v>C1 Полезность — Соу Мамаду</x:v>
+      </x:c>
+      <x:c r="B142" s="4"/>
+      <x:c r="C142" s="4"/>
+      <x:c r="D142" s="4"/>
+      <x:c r="E142" s="4"/>
+      <x:c r="F142" s="4"/>
+      <x:c r="G142" s="4"/>
+      <x:c r="H142" s="4"/>
+      <x:c r="I142" s="4"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B143" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C143" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D143" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E143" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F143" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G143" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H143" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I143" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B144" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C144" s="5" t="n">
+        <x:f>'Оценки'!G47</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D144" s="5" t="n">
+        <x:f>'Оценки'!G48</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E144" s="5" t="n">
+        <x:f>'Оценки'!G49</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F144" s="5" t="n">
+        <x:f>PRODUCT(B144:E144)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G144" s="5" t="n">
+        <x:f>F144/SUM($F$144:$F$147)</x:f>
+        <x:v>0.20529665596111354</x:v>
+      </x:c>
+      <x:c r="H144" s="5" t="n">
+        <x:f>B144*$G$144+C144*$G$145+D144*$G$146+E144*$G$147</x:f>
+        <x:v>0.8273667779387246</x:v>
+      </x:c>
+      <x:c r="I144" s="5" t="n">
+        <x:f>H144/G144</x:f>
+        <x:v>4.030103530256436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B145" s="5" t="n">
+        <x:f>1/C144</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C145" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D145" s="5" t="n">
+        <x:f>'Оценки'!G50</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E145" s="5" t="n">
+        <x:f>'Оценки'!G51</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F145" s="5" t="n">
+        <x:f>PRODUCT(B145:E145)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G145" s="5" t="n">
+        <x:f>F145/SUM($F$144:$F$147)</x:f>
+        <x:v>0.20529665596111354</x:v>
+      </x:c>
+      <x:c r="H145" s="5" t="n">
+        <x:f>B145*$G$144+C145*$G$145+D145*$G$146+E145*$G$147</x:f>
+        <x:v>0.8273667779387246</x:v>
+      </x:c>
+      <x:c r="I145" s="5" t="n">
+        <x:f>H145/G145</x:f>
+        <x:v>4.030103530256436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B146" s="5" t="n">
+        <x:f>1/D144</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C146" s="5" t="n">
+        <x:f>1/D145</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D146" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E146" s="5" t="n">
+        <x:f>'Оценки'!G52</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F146" s="5" t="n">
+        <x:f>PRODUCT(B146:E146)^(1/4)</x:f>
+        <x:v>1.4142135623730951</x:v>
+      </x:c>
+      <x:c r="G146" s="5" t="n">
+        <x:f>F146/SUM($F$144:$F$147)</x:f>
+        <x:v>0.34526644412255103</x:v>
+      </x:c>
+      <x:c r="H146" s="5" t="n">
+        <x:f>B146*$G$144+C146*$G$145+D146*$G$146+E146*$G$147</x:f>
+        <x:v>1.4105933119222271</x:v>
+      </x:c>
+      <x:c r="I146" s="5" t="n">
+        <x:f>H146/G146</x:f>
+        <x:v>4.0855210111919895</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B147" s="5" t="n">
+        <x:f>1/E144</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C147" s="5" t="n">
+        <x:f>1/E145</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D147" s="5" t="n">
+        <x:f>1/E146</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E147" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F147" s="5" t="n">
+        <x:f>PRODUCT(B147:E147)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G147" s="5" t="n">
+        <x:f>F147/SUM($F$144:$F$147)</x:f>
+        <x:v>0.24414024395522202</x:v>
+      </x:c>
+      <x:c r="H147" s="5" t="n">
+        <x:f>B147*$G$144+C147*$G$145+D147*$G$146+E147*$G$147</x:f>
+        <x:v>1.0000000000000002</x:v>
+      </x:c>
+      <x:c r="I147" s="5" t="n">
+        <x:f>H147/G147</x:f>
+        <x:v>4.096006392880525</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="B148" s="5"/>
+      <x:c r="C148" s="5"/>
+      <x:c r="D148" s="5"/>
+      <x:c r="E148" s="5"/>
+      <x:c r="F148" s="5"/>
+      <x:c r="G148" s="5"/>
+      <x:c r="H148" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I148" s="5" t="n">
+        <x:f>AVERAGE(I144:I147)</x:f>
+        <x:v>4.060433616146346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="B149" s="5"/>
+      <x:c r="C149" s="5"/>
+      <x:c r="D149" s="5"/>
+      <x:c r="E149" s="5"/>
+      <x:c r="F149" s="5"/>
+      <x:c r="G149" s="5"/>
+      <x:c r="H149" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I149" s="5" t="n">
+        <x:f>(I148-4)/3</x:f>
+        <x:v>0.020144538715448707</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="B150" s="5"/>
+      <x:c r="C150" s="5"/>
+      <x:c r="D150" s="5"/>
+      <x:c r="E150" s="5"/>
+      <x:c r="F150" s="5"/>
+      <x:c r="G150" s="5"/>
+      <x:c r="H150" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I150" s="5" t="n">
+        <x:f>I149/0.9</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="4" t="str">
+        <x:v>C2 Реализуемость — Роман Иванин</x:v>
+      </x:c>
+      <x:c r="B152" s="4"/>
+      <x:c r="C152" s="4"/>
+      <x:c r="D152" s="4"/>
+      <x:c r="E152" s="4"/>
+      <x:c r="F152" s="4"/>
+      <x:c r="G152" s="4"/>
+      <x:c r="H152" s="4"/>
+      <x:c r="I152" s="4"/>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B153" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C153" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D153" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E153" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F153" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G153" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H153" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I153" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B154" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C154" s="5" t="n">
+        <x:f>'Оценки'!D53</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="D154" s="5" t="n">
+        <x:f>'Оценки'!D54</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E154" s="5" t="n">
+        <x:f>'Оценки'!D55</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F154" s="5" t="n">
+        <x:f>PRODUCT(B154:E154)^(1/4)</x:f>
+        <x:v>0.537284965911771</x:v>
+      </x:c>
+      <x:c r="G154" s="5" t="n">
+        <x:f>F154/SUM($F$154:$F$157)</x:f>
+        <x:v>0.1251952390355543</x:v>
+      </x:c>
+      <x:c r="H154" s="5" t="n">
+        <x:f>B154*$G$154+C154*$G$155+D154*$G$156+E154*$G$157</x:f>
+        <x:v>0.501816361109084</x:v>
+      </x:c>
+      <x:c r="I154" s="5" t="n">
+        <x:f>H154/G154</x:f>
+        <x:v>4.008270322217068</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B155" s="5" t="n">
+        <x:f>1/C154</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C155" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D155" s="5" t="n">
+        <x:f>'Оценки'!D56</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E155" s="5" t="n">
+        <x:f>'Оценки'!D57</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F155" s="5" t="n">
+        <x:f>PRODUCT(B155:E155)^(1/4)</x:f>
+        <x:v>1.5650845800732873</x:v>
+      </x:c>
+      <x:c r="G155" s="5" t="n">
+        <x:f>F155/SUM($F$154:$F$157)</x:f>
+        <x:v>0.36468755045215867</x:v>
+      </x:c>
+      <x:c r="H155" s="5" t="n">
+        <x:f>B155*$G$154+C155*$G$155+D155*$G$156+E155*$G$157</x:f>
+        <x:v>1.48340507363698</x:v>
+      </x:c>
+      <x:c r="I155" s="5" t="n">
+        <x:f>H155/G155</x:f>
+        <x:v>4.067605466097696</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B156" s="5" t="n">
+        <x:f>1/D154</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C156" s="5" t="n">
+        <x:f>1/D155</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D156" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E156" s="5" t="n">
+        <x:f>'Оценки'!D58</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F156" s="5" t="n">
+        <x:f>PRODUCT(B156:E156)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G156" s="5" t="n">
+        <x:f>F156/SUM($F$154:$F$157)</x:f>
+        <x:v>0.2771026149464157</x:v>
+      </x:c>
+      <x:c r="H156" s="5" t="n">
+        <x:f>B156*$G$154+C156*$G$155+D156*$G$156+E156*$G$157</x:f>
+        <x:v>1.1251952390355544</x:v>
+      </x:c>
+      <x:c r="I156" s="5" t="n">
+        <x:f>H156/G156</x:f>
+        <x:v>4.060572431816053</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B157" s="5" t="n">
+        <x:f>1/E154</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C157" s="5" t="n">
+        <x:f>1/E155</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D157" s="5" t="n">
+        <x:f>1/E156</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E157" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F157" s="5" t="n">
+        <x:f>PRODUCT(B157:E157)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G157" s="5" t="n">
+        <x:f>F157/SUM($F$154:$F$157)</x:f>
+        <x:v>0.23301459556587137</x:v>
+      </x:c>
+      <x:c r="H157" s="5" t="n">
+        <x:f>B157*$G$154+C157*$G$155+D157*$G$156+E157*$G$157</x:f>
+        <x:v>0.9428514638094749</x:v>
+      </x:c>
+      <x:c r="I157" s="5" t="n">
+        <x:f>H157/G157</x:f>
+        <x:v>4.046319336862906</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="B158" s="5"/>
+      <x:c r="C158" s="5"/>
+      <x:c r="D158" s="5"/>
+      <x:c r="E158" s="5"/>
+      <x:c r="F158" s="5"/>
+      <x:c r="G158" s="5"/>
+      <x:c r="H158" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I158" s="5" t="n">
+        <x:f>AVERAGE(I154:I157)</x:f>
+        <x:v>4.045691889248431</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="B159" s="5"/>
+      <x:c r="C159" s="5"/>
+      <x:c r="D159" s="5"/>
+      <x:c r="E159" s="5"/>
+      <x:c r="F159" s="5"/>
+      <x:c r="G159" s="5"/>
+      <x:c r="H159" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I159" s="5" t="n">
+        <x:f>(I158-4)/3</x:f>
+        <x:v>0.015230629749477012</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="B160" s="5"/>
+      <x:c r="C160" s="5"/>
+      <x:c r="D160" s="5"/>
+      <x:c r="E160" s="5"/>
+      <x:c r="F160" s="5"/>
+      <x:c r="G160" s="5"/>
+      <x:c r="H160" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I160" s="5" t="n">
+        <x:f>I159/0.9</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" s="4" t="str">
+        <x:v>C2 Реализуемость — Баулин Евгений</x:v>
+      </x:c>
+      <x:c r="B162" s="4"/>
+      <x:c r="C162" s="4"/>
+      <x:c r="D162" s="4"/>
+      <x:c r="E162" s="4"/>
+      <x:c r="F162" s="4"/>
+      <x:c r="G162" s="4"/>
+      <x:c r="H162" s="4"/>
+      <x:c r="I162" s="4"/>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B163" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C163" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D163" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E163" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F163" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G163" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H163" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I163" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B164" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C164" s="5" t="n">
+        <x:f>'Оценки'!E53</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D164" s="5" t="n">
+        <x:f>'Оценки'!E54</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E164" s="5" t="n">
+        <x:f>'Оценки'!E55</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F164" s="5" t="n">
+        <x:f>PRODUCT(B164:E164)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G164" s="5" t="n">
+        <x:f>F164/SUM($F$164:$F$167)</x:f>
+        <x:v>0.2052966559611135</x:v>
+      </x:c>
+      <x:c r="H164" s="5" t="n">
+        <x:f>B164*$G$164+C164*$G$165+D164*$G$166+E164*$G$167</x:f>
+        <x:v>0.8273667779387244</x:v>
+      </x:c>
+      <x:c r="I164" s="5" t="n">
+        <x:f>H164/G164</x:f>
+        <x:v>4.030103530256436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B165" s="5" t="n">
+        <x:f>1/C164</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C165" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D165" s="5" t="n">
+        <x:f>'Оценки'!E56</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E165" s="5" t="n">
+        <x:f>'Оценки'!E57</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F165" s="5" t="n">
+        <x:f>PRODUCT(B165:E165)^(1/4)</x:f>
+        <x:v>1.4142135623730951</x:v>
+      </x:c>
+      <x:c r="G165" s="5" t="n">
+        <x:f>F165/SUM($F$164:$F$167)</x:f>
+        <x:v>0.345266444122551</x:v>
+      </x:c>
+      <x:c r="H165" s="5" t="n">
+        <x:f>B165*$G$164+C165*$G$165+D165*$G$166+E165*$G$167</x:f>
+        <x:v>1.410593311922227</x:v>
+      </x:c>
+      <x:c r="I165" s="5" t="n">
+        <x:f>H165/G165</x:f>
+        <x:v>4.0855210111919895</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B166" s="5" t="n">
+        <x:f>1/D164</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C166" s="5" t="n">
+        <x:f>1/D165</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D166" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E166" s="5" t="n">
+        <x:f>'Оценки'!E58</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F166" s="5" t="n">
+        <x:f>PRODUCT(B166:E166)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G166" s="5" t="n">
+        <x:f>F166/SUM($F$164:$F$167)</x:f>
+        <x:v>0.24414024395522196</x:v>
+      </x:c>
+      <x:c r="H166" s="5" t="n">
+        <x:f>B166*$G$164+C166*$G$165+D166*$G$166+E166*$G$167</x:f>
+        <x:v>0.9999999999999999</x:v>
+      </x:c>
+      <x:c r="I166" s="5" t="n">
+        <x:f>H166/G166</x:f>
+        <x:v>4.096006392880524</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B167" s="5" t="n">
+        <x:f>1/E164</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C167" s="5" t="n">
+        <x:f>1/E165</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D167" s="5" t="n">
+        <x:f>1/E166</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E167" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F167" s="5" t="n">
+        <x:f>PRODUCT(B167:E167)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G167" s="5" t="n">
+        <x:f>F167/SUM($F$164:$F$167)</x:f>
+        <x:v>0.2052966559611135</x:v>
+      </x:c>
+      <x:c r="H167" s="5" t="n">
+        <x:f>B167*$G$164+C167*$G$165+D167*$G$166+E167*$G$167</x:f>
+        <x:v>0.8273667779387244</x:v>
+      </x:c>
+      <x:c r="I167" s="5" t="n">
+        <x:f>H167/G167</x:f>
+        <x:v>4.030103530256436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="B168" s="5"/>
+      <x:c r="C168" s="5"/>
+      <x:c r="D168" s="5"/>
+      <x:c r="E168" s="5"/>
+      <x:c r="F168" s="5"/>
+      <x:c r="G168" s="5"/>
+      <x:c r="H168" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I168" s="5" t="n">
+        <x:f>AVERAGE(I164:I167)</x:f>
+        <x:v>4.060433616146346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="B169" s="5"/>
+      <x:c r="C169" s="5"/>
+      <x:c r="D169" s="5"/>
+      <x:c r="E169" s="5"/>
+      <x:c r="F169" s="5"/>
+      <x:c r="G169" s="5"/>
+      <x:c r="H169" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I169" s="5" t="n">
+        <x:f>(I168-4)/3</x:f>
+        <x:v>0.020144538715448707</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="B170" s="5"/>
+      <x:c r="C170" s="5"/>
+      <x:c r="D170" s="5"/>
+      <x:c r="E170" s="5"/>
+      <x:c r="F170" s="5"/>
+      <x:c r="G170" s="5"/>
+      <x:c r="H170" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I170" s="5" t="n">
+        <x:f>I169/0.9</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="4" t="str">
+        <x:v>C2 Реализуемость — Миленин Никита</x:v>
+      </x:c>
+      <x:c r="B172" s="4"/>
+      <x:c r="C172" s="4"/>
+      <x:c r="D172" s="4"/>
+      <x:c r="E172" s="4"/>
+      <x:c r="F172" s="4"/>
+      <x:c r="G172" s="4"/>
+      <x:c r="H172" s="4"/>
+      <x:c r="I172" s="4"/>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B173" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C173" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D173" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E173" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F173" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G173" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H173" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I173" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B174" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C174" s="5" t="n">
+        <x:f>'Оценки'!F53</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="D174" s="5" t="n">
+        <x:f>'Оценки'!F54</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="E174" s="5" t="n">
+        <x:f>'Оценки'!F55</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F174" s="5" t="n">
+        <x:f>PRODUCT(B174:E174)^(1/4)</x:f>
+        <x:v>0.48549177170732344</x:v>
+      </x:c>
+      <x:c r="G174" s="5" t="n">
+        <x:f>F174/SUM($F$174:$F$177)</x:f>
+        <x:v>0.10893874663644044</x:v>
+      </x:c>
+      <x:c r="H174" s="5" t="n">
+        <x:f>B174*$G$174+C174*$G$175+D174*$G$176+E174*$G$177</x:f>
+        <x:v>0.43740707177215826</x:v>
+      </x:c>
+      <x:c r="I174" s="5" t="n">
+        <x:f>H174/G174</x:f>
+        <x:v>4.015165267431523</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B175" s="5" t="n">
+        <x:f>1/C174</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C175" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D175" s="5" t="n">
+        <x:f>'Оценки'!F56</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E175" s="5" t="n">
+        <x:f>'Оценки'!F57</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F175" s="5" t="n">
+        <x:f>PRODUCT(B175:E175)^(1/4)</x:f>
+        <x:v>1.5650845800732873</x:v>
+      </x:c>
+      <x:c r="G175" s="5" t="n">
+        <x:f>F175/SUM($F$174:$F$177)</x:f>
+        <x:v>0.35118690463818575</x:v>
+      </x:c>
+      <x:c r="H175" s="5" t="n">
+        <x:f>B175*$G$174+C175*$G$175+D175*$G$176+E175*$G$177</x:f>
+        <x:v>1.4065649373600688</x:v>
+      </x:c>
+      <x:c r="I175" s="5" t="n">
+        <x:f>H175/G175</x:f>
+        <x:v>4.005174790925642</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B176" s="5" t="n">
+        <x:f>1/D174</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C176" s="5" t="n">
+        <x:f>1/D175</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D176" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E176" s="5" t="n">
+        <x:f>'Оценки'!F58</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F176" s="5" t="n">
+        <x:f>PRODUCT(B176:E176)^(1/4)</x:f>
+        <x:v>1.5650845800732873</x:v>
+      </x:c>
+      <x:c r="G176" s="5" t="n">
+        <x:f>F176/SUM($F$174:$F$177)</x:f>
+        <x:v>0.35118690463818575</x:v>
+      </x:c>
+      <x:c r="H176" s="5" t="n">
+        <x:f>B176*$G$174+C176*$G$175+D176*$G$176+E176*$G$177</x:f>
+        <x:v>1.4065649373600688</x:v>
+      </x:c>
+      <x:c r="I176" s="5" t="n">
+        <x:f>H176/G176</x:f>
+        <x:v>4.005174790925642</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B177" s="5" t="n">
+        <x:f>1/E174</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C177" s="5" t="n">
+        <x:f>1/E175</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D177" s="5" t="n">
+        <x:f>1/E176</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E177" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F177" s="5" t="n">
+        <x:f>PRODUCT(B177:E177)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G177" s="5" t="n">
+        <x:f>F177/SUM($F$174:$F$177)</x:f>
+        <x:v>0.188687444087188</x:v>
+      </x:c>
+      <x:c r="H177" s="5" t="n">
+        <x:f>B177*$G$174+C177*$G$175+D177*$G$176+E177*$G$177</x:f>
+        <x:v>0.7577518419982546</x:v>
+      </x:c>
+      <x:c r="I177" s="5" t="n">
+        <x:f>H177/G177</x:f>
+        <x:v>4.01591025658345</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="B178" s="5"/>
+      <x:c r="C178" s="5"/>
+      <x:c r="D178" s="5"/>
+      <x:c r="E178" s="5"/>
+      <x:c r="F178" s="5"/>
+      <x:c r="G178" s="5"/>
+      <x:c r="H178" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I178" s="5" t="n">
+        <x:f>AVERAGE(I174:I177)</x:f>
+        <x:v>4.010356276466564</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="B179" s="5"/>
+      <x:c r="C179" s="5"/>
+      <x:c r="D179" s="5"/>
+      <x:c r="E179" s="5"/>
+      <x:c r="F179" s="5"/>
+      <x:c r="G179" s="5"/>
+      <x:c r="H179" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I179" s="5" t="n">
+        <x:f>(I178-4)/3</x:f>
+        <x:v>0.0034520921555213726</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="B180" s="5"/>
+      <x:c r="C180" s="5"/>
+      <x:c r="D180" s="5"/>
+      <x:c r="E180" s="5"/>
+      <x:c r="F180" s="5"/>
+      <x:c r="G180" s="5"/>
+      <x:c r="H180" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I180" s="5" t="n">
+        <x:f>I179/0.9</x:f>
+        <x:v>0.003835657950579303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" s="4" t="str">
+        <x:v>C2 Реализуемость — Соу Мамаду</x:v>
+      </x:c>
+      <x:c r="B182" s="4"/>
+      <x:c r="C182" s="4"/>
+      <x:c r="D182" s="4"/>
+      <x:c r="E182" s="4"/>
+      <x:c r="F182" s="4"/>
+      <x:c r="G182" s="4"/>
+      <x:c r="H182" s="4"/>
+      <x:c r="I182" s="4"/>
+    </x:row>
+    <x:row r="183">
+      <x:c r="A183" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B183" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C183" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D183" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E183" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F183" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G183" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H183" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I183" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B184" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C184" s="5" t="n">
+        <x:f>'Оценки'!G53</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D184" s="5" t="n">
+        <x:f>'Оценки'!G54</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E184" s="5" t="n">
+        <x:f>'Оценки'!G55</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F184" s="5" t="n">
+        <x:f>PRODUCT(B184:E184)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G184" s="5" t="n">
+        <x:f>F184/SUM($F$184:$F$187)</x:f>
+        <x:v>0.2052966559611135</x:v>
+      </x:c>
+      <x:c r="H184" s="5" t="n">
+        <x:f>B184*$G$184+C184*$G$185+D184*$G$186+E184*$G$187</x:f>
+        <x:v>0.8273667779387244</x:v>
+      </x:c>
+      <x:c r="I184" s="5" t="n">
+        <x:f>H184/G184</x:f>
+        <x:v>4.030103530256436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185">
+      <x:c r="A185" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B185" s="5" t="n">
+        <x:f>1/C184</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C185" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D185" s="5" t="n">
+        <x:f>'Оценки'!G56</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E185" s="5" t="n">
+        <x:f>'Оценки'!G57</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F185" s="5" t="n">
+        <x:f>PRODUCT(B185:E185)^(1/4)</x:f>
+        <x:v>1.4142135623730951</x:v>
+      </x:c>
+      <x:c r="G185" s="5" t="n">
+        <x:f>F185/SUM($F$184:$F$187)</x:f>
+        <x:v>0.345266444122551</x:v>
+      </x:c>
+      <x:c r="H185" s="5" t="n">
+        <x:f>B185*$G$184+C185*$G$185+D185*$G$186+E185*$G$187</x:f>
+        <x:v>1.410593311922227</x:v>
+      </x:c>
+      <x:c r="I185" s="5" t="n">
+        <x:f>H185/G185</x:f>
+        <x:v>4.0855210111919895</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186">
+      <x:c r="A186" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B186" s="5" t="n">
+        <x:f>1/D184</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C186" s="5" t="n">
+        <x:f>1/D185</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D186" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E186" s="5" t="n">
+        <x:f>'Оценки'!G58</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F186" s="5" t="n">
+        <x:f>PRODUCT(B186:E186)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G186" s="5" t="n">
+        <x:f>F186/SUM($F$184:$F$187)</x:f>
+        <x:v>0.24414024395522196</x:v>
+      </x:c>
+      <x:c r="H186" s="5" t="n">
+        <x:f>B186*$G$184+C186*$G$185+D186*$G$186+E186*$G$187</x:f>
+        <x:v>0.9999999999999999</x:v>
+      </x:c>
+      <x:c r="I186" s="5" t="n">
+        <x:f>H186/G186</x:f>
+        <x:v>4.096006392880524</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187">
+      <x:c r="A187" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B187" s="5" t="n">
+        <x:f>1/E184</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C187" s="5" t="n">
+        <x:f>1/E185</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D187" s="5" t="n">
+        <x:f>1/E186</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E187" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F187" s="5" t="n">
+        <x:f>PRODUCT(B187:E187)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G187" s="5" t="n">
+        <x:f>F187/SUM($F$184:$F$187)</x:f>
+        <x:v>0.2052966559611135</x:v>
+      </x:c>
+      <x:c r="H187" s="5" t="n">
+        <x:f>B187*$G$184+C187*$G$185+D187*$G$186+E187*$G$187</x:f>
+        <x:v>0.8273667779387244</x:v>
+      </x:c>
+      <x:c r="I187" s="5" t="n">
+        <x:f>H187/G187</x:f>
+        <x:v>4.030103530256436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188">
+      <x:c r="B188" s="5"/>
+      <x:c r="C188" s="5"/>
+      <x:c r="D188" s="5"/>
+      <x:c r="E188" s="5"/>
+      <x:c r="F188" s="5"/>
+      <x:c r="G188" s="5"/>
+      <x:c r="H188" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I188" s="5" t="n">
+        <x:f>AVERAGE(I184:I187)</x:f>
+        <x:v>4.060433616146346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189">
+      <x:c r="B189" s="5"/>
+      <x:c r="C189" s="5"/>
+      <x:c r="D189" s="5"/>
+      <x:c r="E189" s="5"/>
+      <x:c r="F189" s="5"/>
+      <x:c r="G189" s="5"/>
+      <x:c r="H189" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I189" s="5" t="n">
+        <x:f>(I188-4)/3</x:f>
+        <x:v>0.020144538715448707</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190">
+      <x:c r="B190" s="5"/>
+      <x:c r="C190" s="5"/>
+      <x:c r="D190" s="5"/>
+      <x:c r="E190" s="5"/>
+      <x:c r="F190" s="5"/>
+      <x:c r="G190" s="5"/>
+      <x:c r="H190" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I190" s="5" t="n">
+        <x:f>I189/0.9</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192">
+      <x:c r="A192" s="4" t="str">
+        <x:v>C3 Ясность сценариев — Роман Иванин</x:v>
+      </x:c>
+      <x:c r="B192" s="4"/>
+      <x:c r="C192" s="4"/>
+      <x:c r="D192" s="4"/>
+      <x:c r="E192" s="4"/>
+      <x:c r="F192" s="4"/>
+      <x:c r="G192" s="4"/>
+      <x:c r="H192" s="4"/>
+      <x:c r="I192" s="4"/>
+    </x:row>
+    <x:row r="193">
+      <x:c r="A193" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B193" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C193" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D193" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E193" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F193" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G193" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H193" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I193" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194">
+      <x:c r="A194" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B194" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C194" s="5" t="n">
+        <x:f>'Оценки'!D59</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D194" s="5" t="n">
+        <x:f>'Оценки'!D60</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E194" s="5" t="n">
+        <x:f>'Оценки'!D61</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F194" s="5" t="n">
+        <x:f>PRODUCT(B194:E194)^(1/4)</x:f>
+        <x:v>1.5650845800732873</x:v>
+      </x:c>
+      <x:c r="G194" s="5" t="n">
+        <x:f>F194/SUM($F$194:$F$197)</x:f>
+        <x:v>0.35118690463818575</x:v>
+      </x:c>
+      <x:c r="H194" s="5" t="n">
+        <x:f>B194*$G$194+C194*$G$195+D194*$G$196+E194*$G$197</x:f>
+        <x:v>1.4065649373600688</x:v>
+      </x:c>
+      <x:c r="I194" s="5" t="n">
+        <x:f>H194/G194</x:f>
+        <x:v>4.005174790925642</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195">
+      <x:c r="A195" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B195" s="5" t="n">
+        <x:f>1/C194</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="C195" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D195" s="5" t="n">
+        <x:f>'Оценки'!D62</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="E195" s="5" t="n">
+        <x:f>'Оценки'!D63</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F195" s="5" t="n">
+        <x:f>PRODUCT(B195:E195)^(1/4)</x:f>
+        <x:v>0.48549177170732344</x:v>
+      </x:c>
+      <x:c r="G195" s="5" t="n">
+        <x:f>F195/SUM($F$194:$F$197)</x:f>
+        <x:v>0.10893874663644044</x:v>
+      </x:c>
+      <x:c r="H195" s="5" t="n">
+        <x:f>B195*$G$194+C195*$G$195+D195*$G$196+E195*$G$197</x:f>
+        <x:v>0.43740707177215826</x:v>
+      </x:c>
+      <x:c r="I195" s="5" t="n">
+        <x:f>H195/G195</x:f>
+        <x:v>4.015165267431523</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196">
+      <x:c r="A196" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B196" s="5" t="n">
+        <x:f>1/D194</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C196" s="5" t="n">
+        <x:f>1/D195</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D196" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E196" s="5" t="n">
+        <x:f>'Оценки'!D64</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F196" s="5" t="n">
+        <x:f>PRODUCT(B196:E196)^(1/4)</x:f>
+        <x:v>1.5650845800732873</x:v>
+      </x:c>
+      <x:c r="G196" s="5" t="n">
+        <x:f>F196/SUM($F$194:$F$197)</x:f>
+        <x:v>0.35118690463818575</x:v>
+      </x:c>
+      <x:c r="H196" s="5" t="n">
+        <x:f>B196*$G$194+C196*$G$195+D196*$G$196+E196*$G$197</x:f>
+        <x:v>1.4065649373600688</x:v>
+      </x:c>
+      <x:c r="I196" s="5" t="n">
+        <x:f>H196/G196</x:f>
+        <x:v>4.005174790925642</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B197" s="5" t="n">
+        <x:f>1/E194</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C197" s="5" t="n">
+        <x:f>1/E195</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D197" s="5" t="n">
+        <x:f>1/E196</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E197" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F197" s="5" t="n">
+        <x:f>PRODUCT(B197:E197)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G197" s="5" t="n">
+        <x:f>F197/SUM($F$194:$F$197)</x:f>
+        <x:v>0.188687444087188</x:v>
+      </x:c>
+      <x:c r="H197" s="5" t="n">
+        <x:f>B197*$G$194+C197*$G$195+D197*$G$196+E197*$G$197</x:f>
+        <x:v>0.7577518419982546</x:v>
+      </x:c>
+      <x:c r="I197" s="5" t="n">
+        <x:f>H197/G197</x:f>
+        <x:v>4.01591025658345</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198">
+      <x:c r="B198" s="5"/>
+      <x:c r="C198" s="5"/>
+      <x:c r="D198" s="5"/>
+      <x:c r="E198" s="5"/>
+      <x:c r="F198" s="5"/>
+      <x:c r="G198" s="5"/>
+      <x:c r="H198" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I198" s="5" t="n">
+        <x:f>AVERAGE(I194:I197)</x:f>
+        <x:v>4.010356276466564</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199">
+      <x:c r="B199" s="5"/>
+      <x:c r="C199" s="5"/>
+      <x:c r="D199" s="5"/>
+      <x:c r="E199" s="5"/>
+      <x:c r="F199" s="5"/>
+      <x:c r="G199" s="5"/>
+      <x:c r="H199" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I199" s="5" t="n">
+        <x:f>(I198-4)/3</x:f>
+        <x:v>0.0034520921555213726</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200">
+      <x:c r="B200" s="5"/>
+      <x:c r="C200" s="5"/>
+      <x:c r="D200" s="5"/>
+      <x:c r="E200" s="5"/>
+      <x:c r="F200" s="5"/>
+      <x:c r="G200" s="5"/>
+      <x:c r="H200" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I200" s="5" t="n">
+        <x:f>I199/0.9</x:f>
+        <x:v>0.003835657950579303</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" s="4" t="str">
+        <x:v>C3 Ясность сценариев — Баулин Евгений</x:v>
+      </x:c>
+      <x:c r="B202" s="4"/>
+      <x:c r="C202" s="4"/>
+      <x:c r="D202" s="4"/>
+      <x:c r="E202" s="4"/>
+      <x:c r="F202" s="4"/>
+      <x:c r="G202" s="4"/>
+      <x:c r="H202" s="4"/>
+      <x:c r="I202" s="4"/>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B203" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C203" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D203" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E203" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F203" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G203" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H203" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I203" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204">
+      <x:c r="A204" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B204" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C204" s="5" t="n">
+        <x:f>'Оценки'!E59</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D204" s="5" t="n">
+        <x:f>'Оценки'!E60</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E204" s="5" t="n">
+        <x:f>'Оценки'!E61</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F204" s="5" t="n">
+        <x:f>PRODUCT(B204:E204)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G204" s="5" t="n">
+        <x:f>F204/SUM($F$204:$F$207)</x:f>
+        <x:v>0.2771026149464157</x:v>
+      </x:c>
+      <x:c r="H204" s="5" t="n">
+        <x:f>B204*$G$204+C204*$G$205+D204*$G$206+E204*$G$207</x:f>
+        <x:v>1.1251952390355544</x:v>
+      </x:c>
+      <x:c r="I204" s="5" t="n">
+        <x:f>H204/G204</x:f>
+        <x:v>4.060572431816053</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205">
+      <x:c r="A205" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B205" s="5" t="n">
+        <x:f>1/C204</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C205" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D205" s="5" t="n">
+        <x:f>'Оценки'!E62</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="E205" s="5" t="n">
+        <x:f>'Оценки'!E63</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F205" s="5" t="n">
+        <x:f>PRODUCT(B205:E205)^(1/4)</x:f>
+        <x:v>0.537284965911771</x:v>
+      </x:c>
+      <x:c r="G205" s="5" t="n">
+        <x:f>F205/SUM($F$204:$F$207)</x:f>
+        <x:v>0.1251952390355543</x:v>
+      </x:c>
+      <x:c r="H205" s="5" t="n">
+        <x:f>B205*$G$204+C205*$G$205+D205*$G$206+E205*$G$207</x:f>
+        <x:v>0.5018163611090841</x:v>
+      </x:c>
+      <x:c r="I205" s="5" t="n">
+        <x:f>H205/G205</x:f>
+        <x:v>4.008270322217069</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206">
+      <x:c r="A206" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B206" s="5" t="n">
+        <x:f>1/D204</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C206" s="5" t="n">
+        <x:f>1/D205</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D206" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E206" s="5" t="n">
+        <x:f>'Оценки'!E64</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F206" s="5" t="n">
+        <x:f>PRODUCT(B206:E206)^(1/4)</x:f>
+        <x:v>1.5650845800732873</x:v>
+      </x:c>
+      <x:c r="G206" s="5" t="n">
+        <x:f>F206/SUM($F$204:$F$207)</x:f>
+        <x:v>0.36468755045215867</x:v>
+      </x:c>
+      <x:c r="H206" s="5" t="n">
+        <x:f>B206*$G$204+C206*$G$205+D206*$G$206+E206*$G$207</x:f>
+        <x:v>1.48340507363698</x:v>
+      </x:c>
+      <x:c r="I206" s="5" t="n">
+        <x:f>H206/G206</x:f>
+        <x:v>4.067605466097696</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207">
+      <x:c r="A207" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B207" s="5" t="n">
+        <x:f>1/E204</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C207" s="5" t="n">
+        <x:f>1/E205</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D207" s="5" t="n">
+        <x:f>1/E206</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E207" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F207" s="5" t="n">
+        <x:f>PRODUCT(B207:E207)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G207" s="5" t="n">
+        <x:f>F207/SUM($F$204:$F$207)</x:f>
+        <x:v>0.23301459556587137</x:v>
+      </x:c>
+      <x:c r="H207" s="5" t="n">
+        <x:f>B207*$G$204+C207*$G$205+D207*$G$206+E207*$G$207</x:f>
+        <x:v>0.942851463809475</x:v>
+      </x:c>
+      <x:c r="I207" s="5" t="n">
+        <x:f>H207/G207</x:f>
+        <x:v>4.046319336862907</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208">
+      <x:c r="B208" s="5"/>
+      <x:c r="C208" s="5"/>
+      <x:c r="D208" s="5"/>
+      <x:c r="E208" s="5"/>
+      <x:c r="F208" s="5"/>
+      <x:c r="G208" s="5"/>
+      <x:c r="H208" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I208" s="5" t="n">
+        <x:f>AVERAGE(I204:I207)</x:f>
+        <x:v>4.045691889248431</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209">
+      <x:c r="B209" s="5"/>
+      <x:c r="C209" s="5"/>
+      <x:c r="D209" s="5"/>
+      <x:c r="E209" s="5"/>
+      <x:c r="F209" s="5"/>
+      <x:c r="G209" s="5"/>
+      <x:c r="H209" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I209" s="5" t="n">
+        <x:f>(I208-4)/3</x:f>
+        <x:v>0.015230629749477012</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210">
+      <x:c r="B210" s="5"/>
+      <x:c r="C210" s="5"/>
+      <x:c r="D210" s="5"/>
+      <x:c r="E210" s="5"/>
+      <x:c r="F210" s="5"/>
+      <x:c r="G210" s="5"/>
+      <x:c r="H210" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I210" s="5" t="n">
+        <x:f>I209/0.9</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212">
+      <x:c r="A212" s="4" t="str">
+        <x:v>C3 Ясность сценариев — Миленин Никита</x:v>
+      </x:c>
+      <x:c r="B212" s="4"/>
+      <x:c r="C212" s="4"/>
+      <x:c r="D212" s="4"/>
+      <x:c r="E212" s="4"/>
+      <x:c r="F212" s="4"/>
+      <x:c r="G212" s="4"/>
+      <x:c r="H212" s="4"/>
+      <x:c r="I212" s="4"/>
+    </x:row>
+    <x:row r="213">
+      <x:c r="A213" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B213" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C213" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D213" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E213" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F213" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G213" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H213" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I213" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214">
+      <x:c r="A214" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B214" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C214" s="5" t="n">
+        <x:f>'Оценки'!F59</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D214" s="5" t="n">
+        <x:f>'Оценки'!F60</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E214" s="5" t="n">
+        <x:f>'Оценки'!F61</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F214" s="5" t="n">
+        <x:f>PRODUCT(B214:E214)^(1/4)</x:f>
+        <x:v>1.3160740129524924</x:v>
+      </x:c>
+      <x:c r="G214" s="5" t="n">
+        <x:f>F214/SUM($F$214:$F$217)</x:f>
+        <x:v>0.31099823832572826</x:v>
+      </x:c>
+      <x:c r="H214" s="5" t="n">
+        <x:f>B214*$G$214+C214*$G$215+D214*$G$216+E214*$G$217</x:f>
+        <x:v>1.2539289982675033</x:v>
+      </x:c>
+      <x:c r="I214" s="5" t="n">
+        <x:f>H214/G214</x:f>
+        <x:v>4.031948878611279</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215">
+      <x:c r="A215" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B215" s="5" t="n">
+        <x:f>1/C214</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="C215" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D215" s="5" t="n">
+        <x:f>'Оценки'!F62</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E215" s="5" t="n">
+        <x:f>'Оценки'!F63</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F215" s="5" t="n">
+        <x:f>PRODUCT(B215:E215)^(1/4)</x:f>
+        <x:v>0.537284965911771</x:v>
+      </x:c>
+      <x:c r="G215" s="5" t="n">
+        <x:f>F215/SUM($F$214:$F$217)</x:f>
+        <x:v>0.12696449913375163</x:v>
+      </x:c>
+      <x:c r="H215" s="5" t="n">
+        <x:f>B215*$G$214+C215*$G$215+D215*$G$216+E215*$G$217</x:f>
+        <x:v>0.5116492098459211</x:v>
+      </x:c>
+      <x:c r="I215" s="5" t="n">
+        <x:f>H215/G215</x:f>
+        <x:v>4.029860420328369</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216">
+      <x:c r="A216" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B216" s="5" t="n">
+        <x:f>1/D214</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C216" s="5" t="n">
+        <x:f>1/D215</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D216" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E216" s="5" t="n">
+        <x:f>'Оценки'!F64</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F216" s="5" t="n">
+        <x:f>PRODUCT(B216:E216)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G216" s="5" t="n">
+        <x:f>F216/SUM($F$214:$F$217)</x:f>
+        <x:v>0.2810186312702601</x:v>
+      </x:c>
+      <x:c r="H216" s="5" t="n">
+        <x:f>B216*$G$214+C216*$G$215+D216*$G$216+E216*$G$217</x:f>
+        <x:v>1.1269644991337517</x:v>
+      </x:c>
+      <x:c r="I216" s="5" t="n">
+        <x:f>H216/G216</x:f>
+        <x:v>4.010283923310166</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217">
+      <x:c r="A217" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B217" s="5" t="n">
+        <x:f>1/E214</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C217" s="5" t="n">
+        <x:f>1/E215</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D217" s="5" t="n">
+        <x:f>1/E216</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E217" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F217" s="5" t="n">
+        <x:f>PRODUCT(B217:E217)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G217" s="5" t="n">
+        <x:f>F217/SUM($F$214:$F$217)</x:f>
+        <x:v>0.2810186312702601</x:v>
+      </x:c>
+      <x:c r="H217" s="5" t="n">
+        <x:f>B217*$G$214+C217*$G$215+D217*$G$216+E217*$G$217</x:f>
+        <x:v>1.1269644991337517</x:v>
+      </x:c>
+      <x:c r="I217" s="5" t="n">
+        <x:f>H217/G217</x:f>
+        <x:v>4.010283923310166</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218">
+      <x:c r="B218" s="5"/>
+      <x:c r="C218" s="5"/>
+      <x:c r="D218" s="5"/>
+      <x:c r="E218" s="5"/>
+      <x:c r="F218" s="5"/>
+      <x:c r="G218" s="5"/>
+      <x:c r="H218" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I218" s="5" t="n">
+        <x:f>AVERAGE(I214:I217)</x:f>
+        <x:v>4.020594286389994</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219">
+      <x:c r="B219" s="5"/>
+      <x:c r="C219" s="5"/>
+      <x:c r="D219" s="5"/>
+      <x:c r="E219" s="5"/>
+      <x:c r="F219" s="5"/>
+      <x:c r="G219" s="5"/>
+      <x:c r="H219" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I219" s="5" t="n">
+        <x:f>(I218-4)/3</x:f>
+        <x:v>0.006864762129998129</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220">
+      <x:c r="B220" s="5"/>
+      <x:c r="C220" s="5"/>
+      <x:c r="D220" s="5"/>
+      <x:c r="E220" s="5"/>
+      <x:c r="F220" s="5"/>
+      <x:c r="G220" s="5"/>
+      <x:c r="H220" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I220" s="5" t="n">
+        <x:f>I219/0.9</x:f>
+        <x:v>0.007627513477775699</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222">
+      <x:c r="A222" s="4" t="str">
+        <x:v>C3 Ясность сценариев — Соу Мамаду</x:v>
+      </x:c>
+      <x:c r="B222" s="4"/>
+      <x:c r="C222" s="4"/>
+      <x:c r="D222" s="4"/>
+      <x:c r="E222" s="4"/>
+      <x:c r="F222" s="4"/>
+      <x:c r="G222" s="4"/>
+      <x:c r="H222" s="4"/>
+      <x:c r="I222" s="4"/>
+    </x:row>
+    <x:row r="223">
+      <x:c r="A223" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B223" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C223" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D223" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E223" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F223" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G223" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H223" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I223" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224">
+      <x:c r="A224" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B224" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C224" s="5" t="n">
+        <x:f>'Оценки'!G59</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D224" s="5" t="n">
+        <x:f>'Оценки'!G60</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E224" s="5" t="n">
+        <x:f>'Оценки'!G61</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F224" s="5" t="n">
+        <x:f>PRODUCT(B224:E224)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G224" s="5" t="n">
+        <x:f>F224/SUM($F$224:$F$227)</x:f>
+        <x:v>0.24414024395522196</x:v>
+      </x:c>
+      <x:c r="H224" s="5" t="n">
+        <x:f>B224*$G$224+C224*$G$225+D224*$G$226+E224*$G$227</x:f>
+        <x:v>0.9999999999999999</x:v>
+      </x:c>
+      <x:c r="I224" s="5" t="n">
+        <x:f>H224/G224</x:f>
+        <x:v>4.096006392880524</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225">
+      <x:c r="A225" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B225" s="5" t="n">
+        <x:f>1/C224</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C225" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D225" s="5" t="n">
+        <x:f>'Оценки'!G62</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E225" s="5" t="n">
+        <x:f>'Оценки'!G63</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F225" s="5" t="n">
+        <x:f>PRODUCT(B225:E225)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G225" s="5" t="n">
+        <x:f>F225/SUM($F$224:$F$227)</x:f>
+        <x:v>0.2052966559611135</x:v>
+      </x:c>
+      <x:c r="H225" s="5" t="n">
+        <x:f>B225*$G$224+C225*$G$225+D225*$G$226+E225*$G$227</x:f>
+        <x:v>0.8273667779387244</x:v>
+      </x:c>
+      <x:c r="I225" s="5" t="n">
+        <x:f>H225/G225</x:f>
+        <x:v>4.030103530256436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226">
+      <x:c r="A226" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B226" s="5" t="n">
+        <x:f>1/D224</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C226" s="5" t="n">
+        <x:f>1/D225</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D226" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E226" s="5" t="n">
+        <x:f>'Оценки'!G64</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F226" s="5" t="n">
+        <x:f>PRODUCT(B226:E226)^(1/4)</x:f>
+        <x:v>1.4142135623730951</x:v>
+      </x:c>
+      <x:c r="G226" s="5" t="n">
+        <x:f>F226/SUM($F$224:$F$227)</x:f>
+        <x:v>0.345266444122551</x:v>
+      </x:c>
+      <x:c r="H226" s="5" t="n">
+        <x:f>B226*$G$224+C226*$G$225+D226*$G$226+E226*$G$227</x:f>
+        <x:v>1.410593311922227</x:v>
+      </x:c>
+      <x:c r="I226" s="5" t="n">
+        <x:f>H226/G226</x:f>
+        <x:v>4.0855210111919895</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227">
+      <x:c r="A227" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B227" s="5" t="n">
+        <x:f>1/E224</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C227" s="5" t="n">
+        <x:f>1/E225</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D227" s="5" t="n">
+        <x:f>1/E226</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E227" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F227" s="5" t="n">
+        <x:f>PRODUCT(B227:E227)^(1/4)</x:f>
+        <x:v>0.8408964152537145</x:v>
+      </x:c>
+      <x:c r="G227" s="5" t="n">
+        <x:f>F227/SUM($F$224:$F$227)</x:f>
+        <x:v>0.2052966559611135</x:v>
+      </x:c>
+      <x:c r="H227" s="5" t="n">
+        <x:f>B227*$G$224+C227*$G$225+D227*$G$226+E227*$G$227</x:f>
+        <x:v>0.8273667779387244</x:v>
+      </x:c>
+      <x:c r="I227" s="5" t="n">
+        <x:f>H227/G227</x:f>
+        <x:v>4.030103530256436</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228">
+      <x:c r="B228" s="5"/>
+      <x:c r="C228" s="5"/>
+      <x:c r="D228" s="5"/>
+      <x:c r="E228" s="5"/>
+      <x:c r="F228" s="5"/>
+      <x:c r="G228" s="5"/>
+      <x:c r="H228" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I228" s="5" t="n">
+        <x:f>AVERAGE(I224:I227)</x:f>
+        <x:v>4.060433616146346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229">
+      <x:c r="B229" s="5"/>
+      <x:c r="C229" s="5"/>
+      <x:c r="D229" s="5"/>
+      <x:c r="E229" s="5"/>
+      <x:c r="F229" s="5"/>
+      <x:c r="G229" s="5"/>
+      <x:c r="H229" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I229" s="5" t="n">
+        <x:f>(I228-4)/3</x:f>
+        <x:v>0.020144538715448707</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230">
+      <x:c r="B230" s="5"/>
+      <x:c r="C230" s="5"/>
+      <x:c r="D230" s="5"/>
+      <x:c r="E230" s="5"/>
+      <x:c r="F230" s="5"/>
+      <x:c r="G230" s="5"/>
+      <x:c r="H230" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I230" s="5" t="n">
+        <x:f>I229/0.9</x:f>
+        <x:v>0.02238282079494301</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232">
+      <x:c r="A232" s="4" t="str">
+        <x:v>C4 Пригодность для планирования — Роман Иванин</x:v>
+      </x:c>
+      <x:c r="B232" s="4"/>
+      <x:c r="C232" s="4"/>
+      <x:c r="D232" s="4"/>
+      <x:c r="E232" s="4"/>
+      <x:c r="F232" s="4"/>
+      <x:c r="G232" s="4"/>
+      <x:c r="H232" s="4"/>
+      <x:c r="I232" s="4"/>
+    </x:row>
+    <x:row r="233">
+      <x:c r="A233" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B233" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C233" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D233" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E233" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F233" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G233" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H233" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I233" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234">
+      <x:c r="A234" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B234" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C234" s="5" t="n">
+        <x:f>'Оценки'!D65</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D234" s="5" t="n">
+        <x:f>'Оценки'!D66</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E234" s="5" t="n">
+        <x:f>'Оценки'!D67</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F234" s="5" t="n">
+        <x:f>PRODUCT(B234:E234)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G234" s="5" t="n">
+        <x:f>F234/SUM($F$234:$F$237)</x:f>
+        <x:v>0.23301459556587137</x:v>
+      </x:c>
+      <x:c r="H234" s="5" t="n">
+        <x:f>B234*$G$234+C234*$G$235+D234*$G$236+E234*$G$237</x:f>
+        <x:v>0.942851463809475</x:v>
+      </x:c>
+      <x:c r="I234" s="5" t="n">
+        <x:f>H234/G234</x:f>
+        <x:v>4.046319336862907</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235">
+      <x:c r="A235" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B235" s="5" t="n">
+        <x:f>1/C234</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C235" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D235" s="5" t="n">
+        <x:f>'Оценки'!D68</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E235" s="5" t="n">
+        <x:f>'Оценки'!D69</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="F235" s="5" t="n">
+        <x:f>PRODUCT(B235:E235)^(1/4)</x:f>
+        <x:v>0.537284965911771</x:v>
+      </x:c>
+      <x:c r="G235" s="5" t="n">
+        <x:f>F235/SUM($F$234:$F$237)</x:f>
+        <x:v>0.1251952390355543</x:v>
+      </x:c>
+      <x:c r="H235" s="5" t="n">
+        <x:f>B235*$G$234+C235*$G$235+D235*$G$236+E235*$G$237</x:f>
+        <x:v>0.501816361109084</x:v>
+      </x:c>
+      <x:c r="I235" s="5" t="n">
+        <x:f>H235/G235</x:f>
+        <x:v>4.008270322217068</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236">
+      <x:c r="A236" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B236" s="5" t="n">
+        <x:f>1/D234</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C236" s="5" t="n">
+        <x:f>1/D235</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D236" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E236" s="5" t="n">
+        <x:f>'Оценки'!D70</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F236" s="5" t="n">
+        <x:f>PRODUCT(B236:E236)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G236" s="5" t="n">
+        <x:f>F236/SUM($F$234:$F$237)</x:f>
+        <x:v>0.2771026149464157</x:v>
+      </x:c>
+      <x:c r="H236" s="5" t="n">
+        <x:f>B236*$G$234+C236*$G$235+D236*$G$236+E236*$G$237</x:f>
+        <x:v>1.1251952390355544</x:v>
+      </x:c>
+      <x:c r="I236" s="5" t="n">
+        <x:f>H236/G236</x:f>
+        <x:v>4.060572431816053</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237">
+      <x:c r="A237" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B237" s="5" t="n">
+        <x:f>1/E234</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C237" s="5" t="n">
+        <x:f>1/E235</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D237" s="5" t="n">
+        <x:f>1/E236</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E237" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F237" s="5" t="n">
+        <x:f>PRODUCT(B237:E237)^(1/4)</x:f>
+        <x:v>1.5650845800732873</x:v>
+      </x:c>
+      <x:c r="G237" s="5" t="n">
+        <x:f>F237/SUM($F$234:$F$237)</x:f>
+        <x:v>0.36468755045215867</x:v>
+      </x:c>
+      <x:c r="H237" s="5" t="n">
+        <x:f>B237*$G$234+C237*$G$235+D237*$G$236+E237*$G$237</x:f>
+        <x:v>1.4834050736369802</x:v>
+      </x:c>
+      <x:c r="I237" s="5" t="n">
+        <x:f>H237/G237</x:f>
+        <x:v>4.067605466097697</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238">
+      <x:c r="B238" s="5"/>
+      <x:c r="C238" s="5"/>
+      <x:c r="D238" s="5"/>
+      <x:c r="E238" s="5"/>
+      <x:c r="F238" s="5"/>
+      <x:c r="G238" s="5"/>
+      <x:c r="H238" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I238" s="5" t="n">
+        <x:f>AVERAGE(I234:I237)</x:f>
+        <x:v>4.045691889248431</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239">
+      <x:c r="B239" s="5"/>
+      <x:c r="C239" s="5"/>
+      <x:c r="D239" s="5"/>
+      <x:c r="E239" s="5"/>
+      <x:c r="F239" s="5"/>
+      <x:c r="G239" s="5"/>
+      <x:c r="H239" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I239" s="5" t="n">
+        <x:f>(I238-4)/3</x:f>
+        <x:v>0.015230629749477012</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240">
+      <x:c r="B240" s="5"/>
+      <x:c r="C240" s="5"/>
+      <x:c r="D240" s="5"/>
+      <x:c r="E240" s="5"/>
+      <x:c r="F240" s="5"/>
+      <x:c r="G240" s="5"/>
+      <x:c r="H240" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I240" s="5" t="n">
+        <x:f>I239/0.9</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242">
+      <x:c r="A242" s="4" t="str">
+        <x:v>C4 Пригодность для планирования — Баулин Евгений</x:v>
+      </x:c>
+      <x:c r="B242" s="4"/>
+      <x:c r="C242" s="4"/>
+      <x:c r="D242" s="4"/>
+      <x:c r="E242" s="4"/>
+      <x:c r="F242" s="4"/>
+      <x:c r="G242" s="4"/>
+      <x:c r="H242" s="4"/>
+      <x:c r="I242" s="4"/>
+    </x:row>
+    <x:row r="243">
+      <x:c r="A243" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B243" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C243" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D243" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E243" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F243" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G243" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H243" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I243" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244">
+      <x:c r="A244" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B244" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C244" s="5" t="n">
+        <x:f>'Оценки'!E65</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D244" s="5" t="n">
+        <x:f>'Оценки'!E66</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E244" s="5" t="n">
+        <x:f>'Оценки'!E67</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F244" s="5" t="n">
+        <x:f>PRODUCT(B244:E244)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G244" s="5" t="n">
+        <x:f>F244/SUM($F$244:$F$247)</x:f>
+        <x:v>0.28571428571428575</x:v>
+      </x:c>
+      <x:c r="H244" s="5" t="n">
+        <x:f>B244*$G$244+C244*$G$245+D244*$G$246+E244*$G$247</x:f>
+        <x:v>1.142857142857143</x:v>
+      </x:c>
+      <x:c r="I244" s="5" t="n">
+        <x:f>H244/G244</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245">
+      <x:c r="A245" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B245" s="5" t="n">
+        <x:f>1/C244</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C245" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D245" s="5" t="n">
+        <x:f>'Оценки'!E68</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E245" s="5" t="n">
+        <x:f>'Оценки'!E69</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F245" s="5" t="n">
+        <x:f>PRODUCT(B245:E245)^(1/4)</x:f>
+        <x:v>0.5946035575013605</x:v>
+      </x:c>
+      <x:c r="G245" s="5" t="n">
+        <x:f>F245/SUM($F$244:$F$247)</x:f>
+        <x:v>0.14285714285714288</x:v>
+      </x:c>
+      <x:c r="H245" s="5" t="n">
+        <x:f>B245*$G$244+C245*$G$245+D245*$G$246+E245*$G$247</x:f>
+        <x:v>0.5714285714285715</x:v>
+      </x:c>
+      <x:c r="I245" s="5" t="n">
+        <x:f>H245/G245</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246">
+      <x:c r="A246" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B246" s="5" t="n">
+        <x:f>1/D244</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C246" s="5" t="n">
+        <x:f>1/D245</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D246" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E246" s="5" t="n">
+        <x:f>'Оценки'!E70</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F246" s="5" t="n">
+        <x:f>PRODUCT(B246:E246)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G246" s="5" t="n">
+        <x:f>F246/SUM($F$244:$F$247)</x:f>
+        <x:v>0.28571428571428575</x:v>
+      </x:c>
+      <x:c r="H246" s="5" t="n">
+        <x:f>B246*$G$244+C246*$G$245+D246*$G$246+E246*$G$247</x:f>
+        <x:v>1.142857142857143</x:v>
+      </x:c>
+      <x:c r="I246" s="5" t="n">
+        <x:f>H246/G246</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247">
+      <x:c r="A247" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B247" s="5" t="n">
+        <x:f>1/E244</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C247" s="5" t="n">
+        <x:f>1/E245</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D247" s="5" t="n">
+        <x:f>1/E246</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E247" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F247" s="5" t="n">
+        <x:f>PRODUCT(B247:E247)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G247" s="5" t="n">
+        <x:f>F247/SUM($F$244:$F$247)</x:f>
+        <x:v>0.28571428571428575</x:v>
+      </x:c>
+      <x:c r="H247" s="5" t="n">
+        <x:f>B247*$G$244+C247*$G$245+D247*$G$246+E247*$G$247</x:f>
+        <x:v>1.142857142857143</x:v>
+      </x:c>
+      <x:c r="I247" s="5" t="n">
+        <x:f>H247/G247</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248">
+      <x:c r="B248" s="5"/>
+      <x:c r="C248" s="5"/>
+      <x:c r="D248" s="5"/>
+      <x:c r="E248" s="5"/>
+      <x:c r="F248" s="5"/>
+      <x:c r="G248" s="5"/>
+      <x:c r="H248" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I248" s="5" t="n">
+        <x:f>AVERAGE(I244:I247)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249">
+      <x:c r="B249" s="5"/>
+      <x:c r="C249" s="5"/>
+      <x:c r="D249" s="5"/>
+      <x:c r="E249" s="5"/>
+      <x:c r="F249" s="5"/>
+      <x:c r="G249" s="5"/>
+      <x:c r="H249" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I249" s="5" t="n">
+        <x:f>(I248-4)/3</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250">
+      <x:c r="B250" s="5"/>
+      <x:c r="C250" s="5"/>
+      <x:c r="D250" s="5"/>
+      <x:c r="E250" s="5"/>
+      <x:c r="F250" s="5"/>
+      <x:c r="G250" s="5"/>
+      <x:c r="H250" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I250" s="5" t="n">
+        <x:f>I249/0.9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252">
+      <x:c r="A252" s="4" t="str">
+        <x:v>C4 Пригодность для планирования — Миленин Никита</x:v>
+      </x:c>
+      <x:c r="B252" s="4"/>
+      <x:c r="C252" s="4"/>
+      <x:c r="D252" s="4"/>
+      <x:c r="E252" s="4"/>
+      <x:c r="F252" s="4"/>
+      <x:c r="G252" s="4"/>
+      <x:c r="H252" s="4"/>
+      <x:c r="I252" s="4"/>
+    </x:row>
+    <x:row r="253">
+      <x:c r="A253" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B253" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C253" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D253" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E253" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F253" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G253" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H253" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I253" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254">
+      <x:c r="A254" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B254" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C254" s="5" t="n">
+        <x:f>'Оценки'!F65</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D254" s="5" t="n">
+        <x:f>'Оценки'!F66</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E254" s="5" t="n">
+        <x:f>'Оценки'!F67</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F254" s="5" t="n">
+        <x:f>PRODUCT(B254:E254)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G254" s="5" t="n">
+        <x:f>F254/SUM($F$254:$F$257)</x:f>
+        <x:v>0.23301459556587137</x:v>
+      </x:c>
+      <x:c r="H254" s="5" t="n">
+        <x:f>B254*$G$254+C254*$G$255+D254*$G$256+E254*$G$257</x:f>
+        <x:v>0.942851463809475</x:v>
+      </x:c>
+      <x:c r="I254" s="5" t="n">
+        <x:f>H254/G254</x:f>
+        <x:v>4.046319336862907</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="255">
+      <x:c r="A255" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B255" s="5" t="n">
+        <x:f>1/C254</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C255" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D255" s="5" t="n">
+        <x:f>'Оценки'!F68</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E255" s="5" t="n">
+        <x:f>'Оценки'!F69</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="F255" s="5" t="n">
+        <x:f>PRODUCT(B255:E255)^(1/4)</x:f>
+        <x:v>0.537284965911771</x:v>
+      </x:c>
+      <x:c r="G255" s="5" t="n">
+        <x:f>F255/SUM($F$254:$F$257)</x:f>
+        <x:v>0.1251952390355543</x:v>
+      </x:c>
+      <x:c r="H255" s="5" t="n">
+        <x:f>B255*$G$254+C255*$G$255+D255*$G$256+E255*$G$257</x:f>
+        <x:v>0.501816361109084</x:v>
+      </x:c>
+      <x:c r="I255" s="5" t="n">
+        <x:f>H255/G255</x:f>
+        <x:v>4.008270322217068</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256">
+      <x:c r="A256" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B256" s="5" t="n">
+        <x:f>1/D254</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C256" s="5" t="n">
+        <x:f>1/D255</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D256" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E256" s="5" t="n">
+        <x:f>'Оценки'!F70</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F256" s="5" t="n">
+        <x:f>PRODUCT(B256:E256)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G256" s="5" t="n">
+        <x:f>F256/SUM($F$254:$F$257)</x:f>
+        <x:v>0.2771026149464157</x:v>
+      </x:c>
+      <x:c r="H256" s="5" t="n">
+        <x:f>B256*$G$254+C256*$G$255+D256*$G$256+E256*$G$257</x:f>
+        <x:v>1.1251952390355544</x:v>
+      </x:c>
+      <x:c r="I256" s="5" t="n">
+        <x:f>H256/G256</x:f>
+        <x:v>4.060572431816053</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257">
+      <x:c r="A257" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B257" s="5" t="n">
+        <x:f>1/E254</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C257" s="5" t="n">
+        <x:f>1/E255</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D257" s="5" t="n">
+        <x:f>1/E256</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E257" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F257" s="5" t="n">
+        <x:f>PRODUCT(B257:E257)^(1/4)</x:f>
+        <x:v>1.5650845800732873</x:v>
+      </x:c>
+      <x:c r="G257" s="5" t="n">
+        <x:f>F257/SUM($F$254:$F$257)</x:f>
+        <x:v>0.36468755045215867</x:v>
+      </x:c>
+      <x:c r="H257" s="5" t="n">
+        <x:f>B257*$G$254+C257*$G$255+D257*$G$256+E257*$G$257</x:f>
+        <x:v>1.4834050736369802</x:v>
+      </x:c>
+      <x:c r="I257" s="5" t="n">
+        <x:f>H257/G257</x:f>
+        <x:v>4.067605466097697</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258">
+      <x:c r="B258" s="5"/>
+      <x:c r="C258" s="5"/>
+      <x:c r="D258" s="5"/>
+      <x:c r="E258" s="5"/>
+      <x:c r="F258" s="5"/>
+      <x:c r="G258" s="5"/>
+      <x:c r="H258" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I258" s="5" t="n">
+        <x:f>AVERAGE(I254:I257)</x:f>
+        <x:v>4.045691889248431</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259">
+      <x:c r="B259" s="5"/>
+      <x:c r="C259" s="5"/>
+      <x:c r="D259" s="5"/>
+      <x:c r="E259" s="5"/>
+      <x:c r="F259" s="5"/>
+      <x:c r="G259" s="5"/>
+      <x:c r="H259" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I259" s="5" t="n">
+        <x:f>(I258-4)/3</x:f>
+        <x:v>0.015230629749477012</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260">
+      <x:c r="B260" s="5"/>
+      <x:c r="C260" s="5"/>
+      <x:c r="D260" s="5"/>
+      <x:c r="E260" s="5"/>
+      <x:c r="F260" s="5"/>
+      <x:c r="G260" s="5"/>
+      <x:c r="H260" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I260" s="5" t="n">
+        <x:f>I259/0.9</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262">
+      <x:c r="A262" s="4" t="str">
+        <x:v>C4 Пригодность для планирования — Соу Мамаду</x:v>
+      </x:c>
+      <x:c r="B262" s="4"/>
+      <x:c r="C262" s="4"/>
+      <x:c r="D262" s="4"/>
+      <x:c r="E262" s="4"/>
+      <x:c r="F262" s="4"/>
+      <x:c r="G262" s="4"/>
+      <x:c r="H262" s="4"/>
+      <x:c r="I262" s="4"/>
+    </x:row>
+    <x:row r="263">
+      <x:c r="A263" s="8" t="str">
+        <x:v>Элемент</x:v>
+      </x:c>
+      <x:c r="B263" s="8" t="str">
+        <x:v>A1</x:v>
+      </x:c>
+      <x:c r="C263" s="8" t="str">
+        <x:v>A2</x:v>
+      </x:c>
+      <x:c r="D263" s="8" t="str">
+        <x:v>A3</x:v>
+      </x:c>
+      <x:c r="E263" s="8" t="str">
+        <x:v>A4</x:v>
+      </x:c>
+      <x:c r="F263" s="8" t="str">
+        <x:v>Геом. ср.</x:v>
+      </x:c>
+      <x:c r="G263" s="8" t="str">
+        <x:v>Приоритет</x:v>
+      </x:c>
+      <x:c r="H263" s="8" t="str">
+        <x:v>Aw</x:v>
+      </x:c>
+      <x:c r="I263" s="8" t="str">
+        <x:v>Aw/w</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264">
+      <x:c r="A264" t="str">
+        <x:v>A1 Бронирование помещений</x:v>
+      </x:c>
+      <x:c r="B264" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C264" s="5" t="n">
+        <x:f>'Оценки'!G65</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D264" s="5" t="n">
+        <x:f>'Оценки'!G66</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E264" s="5" t="n">
+        <x:f>'Оценки'!G67</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="F264" s="5" t="n">
+        <x:f>PRODUCT(B264:E264)^(1/4)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G264" s="5" t="n">
+        <x:f>F264/SUM($F$264:$F$267)</x:f>
+        <x:v>0.23301459556587137</x:v>
+      </x:c>
+      <x:c r="H264" s="5" t="n">
+        <x:f>B264*$G$264+C264*$G$265+D264*$G$266+E264*$G$267</x:f>
+        <x:v>0.942851463809475</x:v>
+      </x:c>
+      <x:c r="I264" s="5" t="n">
+        <x:f>H264/G264</x:f>
+        <x:v>4.046319336862907</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265">
+      <x:c r="A265" t="str">
+        <x:v>A2 Учебные группы</x:v>
+      </x:c>
+      <x:c r="B265" s="5" t="n">
+        <x:f>1/C264</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C265" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D265" s="5" t="n">
+        <x:f>'Оценки'!G68</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E265" s="5" t="n">
+        <x:f>'Оценки'!G69</x:f>
+        <x:v>0.3333333333333333</x:v>
+      </x:c>
+      <x:c r="F265" s="5" t="n">
+        <x:f>PRODUCT(B265:E265)^(1/4)</x:f>
+        <x:v>0.537284965911771</x:v>
+      </x:c>
+      <x:c r="G265" s="5" t="n">
+        <x:f>F265/SUM($F$264:$F$267)</x:f>
+        <x:v>0.1251952390355543</x:v>
+      </x:c>
+      <x:c r="H265" s="5" t="n">
+        <x:f>B265*$G$264+C265*$G$265+D265*$G$266+E265*$G$267</x:f>
+        <x:v>0.501816361109084</x:v>
+      </x:c>
+      <x:c r="I265" s="5" t="n">
+        <x:f>H265/G265</x:f>
+        <x:v>4.008270322217068</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266">
+      <x:c r="A266" t="str">
+        <x:v>A3 Студенческие события</x:v>
+      </x:c>
+      <x:c r="B266" s="5" t="n">
+        <x:f>1/D264</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C266" s="5" t="n">
+        <x:f>1/D265</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D266" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E266" s="5" t="n">
+        <x:f>'Оценки'!G70</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F266" s="5" t="n">
+        <x:f>PRODUCT(B266:E266)^(1/4)</x:f>
+        <x:v>1.189207115002721</x:v>
+      </x:c>
+      <x:c r="G266" s="5" t="n">
+        <x:f>F266/SUM($F$264:$F$267)</x:f>
+        <x:v>0.2771026149464157</x:v>
+      </x:c>
+      <x:c r="H266" s="5" t="n">
+        <x:f>B266*$G$264+C266*$G$265+D266*$G$266+E266*$G$267</x:f>
+        <x:v>1.1251952390355544</x:v>
+      </x:c>
+      <x:c r="I266" s="5" t="n">
+        <x:f>H266/G266</x:f>
+        <x:v>4.060572431816053</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267">
+      <x:c r="A267" t="str">
+        <x:v>A4 Волонтёрские смены</x:v>
+      </x:c>
+      <x:c r="B267" s="5" t="n">
+        <x:f>1/E264</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C267" s="5" t="n">
+        <x:f>1/E265</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D267" s="5" t="n">
+        <x:f>1/E266</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E267" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F267" s="5" t="n">
+        <x:f>PRODUCT(B267:E267)^(1/4)</x:f>
+        <x:v>1.5650845800732873</x:v>
+      </x:c>
+      <x:c r="G267" s="5" t="n">
+        <x:f>F267/SUM($F$264:$F$267)</x:f>
+        <x:v>0.36468755045215867</x:v>
+      </x:c>
+      <x:c r="H267" s="5" t="n">
+        <x:f>B267*$G$264+C267*$G$265+D267*$G$266+E267*$G$267</x:f>
+        <x:v>1.4834050736369802</x:v>
+      </x:c>
+      <x:c r="I267" s="5" t="n">
+        <x:f>H267/G267</x:f>
+        <x:v>4.067605466097697</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268">
+      <x:c r="B268" s="5"/>
+      <x:c r="C268" s="5"/>
+      <x:c r="D268" s="5"/>
+      <x:c r="E268" s="5"/>
+      <x:c r="F268" s="5"/>
+      <x:c r="G268" s="5"/>
+      <x:c r="H268" s="5" t="str">
+        <x:v>λmax</x:v>
+      </x:c>
+      <x:c r="I268" s="5" t="n">
+        <x:f>AVERAGE(I264:I267)</x:f>
+        <x:v>4.045691889248431</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269">
+      <x:c r="B269" s="5"/>
+      <x:c r="C269" s="5"/>
+      <x:c r="D269" s="5"/>
+      <x:c r="E269" s="5"/>
+      <x:c r="F269" s="5"/>
+      <x:c r="G269" s="5"/>
+      <x:c r="H269" s="5" t="str">
+        <x:v>CI</x:v>
+      </x:c>
+      <x:c r="I269" s="5" t="n">
+        <x:f>(I268-4)/3</x:f>
+        <x:v>0.015230629749477012</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270">
+      <x:c r="B270" s="5"/>
+      <x:c r="C270" s="5"/>
+      <x:c r="D270" s="5"/>
+      <x:c r="E270" s="5"/>
+      <x:c r="F270" s="5"/>
+      <x:c r="G270" s="5"/>
+      <x:c r="H270" s="5" t="str">
+        <x:v>CR</x:v>
+      </x:c>
+      <x:c r="I270" s="5" t="n">
+        <x:f>I269/0.9</x:f>
+        <x:v>0.016922921943863346</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>
@@ -5168,6 +9967,27 @@
     <x:mergeCell ref="A23:I23"/>
     <x:mergeCell ref="A33:I33"/>
     <x:mergeCell ref="A43:I43"/>
+    <x:mergeCell ref="A62:G62"/>
+    <x:mergeCell ref="A72:I72"/>
+    <x:mergeCell ref="A82:I82"/>
+    <x:mergeCell ref="A92:I92"/>
+    <x:mergeCell ref="A102:I102"/>
+    <x:mergeCell ref="A112:I112"/>
+    <x:mergeCell ref="A122:I122"/>
+    <x:mergeCell ref="A132:I132"/>
+    <x:mergeCell ref="A142:I142"/>
+    <x:mergeCell ref="A152:I152"/>
+    <x:mergeCell ref="A162:I162"/>
+    <x:mergeCell ref="A172:I172"/>
+    <x:mergeCell ref="A182:I182"/>
+    <x:mergeCell ref="A192:I192"/>
+    <x:mergeCell ref="A202:I202"/>
+    <x:mergeCell ref="A212:I212"/>
+    <x:mergeCell ref="A222:I222"/>
+    <x:mergeCell ref="A232:I232"/>
+    <x:mergeCell ref="A242:I242"/>
+    <x:mergeCell ref="A252:I252"/>
+    <x:mergeCell ref="A262:I262"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>